<commit_message>
Per-muscle body diagram in Gym history
Each exercise now lights only the muscles it works (EX_MUSCLES map) instead of whole category zones. Fallback to zone for custom exercises. No data migration needed.
</commit_message>
<xml_diff>
--- a/My Lattice&Climbing training docs/Jo_training raw docs 25_2026/myGym Training 24_2025.xlsx
+++ b/My Lattice&Climbing training docs/Jo_training raw docs 25_2026/myGym Training 24_2025.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/josinabernardes/Documents/My Lattice&amp;Climbing training docs/Jo_training raw docs 25_2026/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/josinabernardes/Documents/Tennis-Tracker-Hub/My Lattice&amp;Climbing training docs/Jo_training raw docs 25_2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99709BE8-A6DA-974B-81D9-B17B69200786}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51EE60B5-5420-874F-9FBF-D6EB1779B797}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4320" yWindow="600" windowWidth="24480" windowHeight="15940" tabRatio="765" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,50 +22,50 @@
   </sheets>
   <definedNames>
     <definedName name="_xlchart.v2.0" hidden="1">'My Climb Log Aug25'!$L$58:$L$65</definedName>
-    <definedName name="_xlchart.v2.1" hidden="1">'My Climb Log Aug25'!$M$57</definedName>
-    <definedName name="_xlchart.v2.10" hidden="1">'My ClimbRecov24_25'!$M$229</definedName>
-    <definedName name="_xlchart.v2.11" hidden="1">'My ClimbRecov24_25'!$M$230:$M$237</definedName>
-    <definedName name="_xlchart.v2.12" hidden="1">'My ClimbRecov24_25'!$L$302:$L$309</definedName>
-    <definedName name="_xlchart.v2.13" hidden="1">'My ClimbRecov24_25'!$N$301</definedName>
-    <definedName name="_xlchart.v2.14" hidden="1">'My ClimbRecov24_25'!$N$302:$N$309</definedName>
-    <definedName name="_xlchart.v2.15" hidden="1">'My ClimbRecov24_25'!$L$302:$L$309</definedName>
-    <definedName name="_xlchart.v2.16" hidden="1">'My ClimbRecov24_25'!$M$302:$M$309</definedName>
-    <definedName name="_xlchart.v2.17" hidden="1">'My ClimbRecov24_25'!$L$88:$L$95</definedName>
-    <definedName name="_xlchart.v2.18" hidden="1">'My ClimbRecov24_25'!$N$87</definedName>
-    <definedName name="_xlchart.v2.19" hidden="1">'My ClimbRecov24_25'!$N$88:$N$95</definedName>
-    <definedName name="_xlchart.v2.2" hidden="1">'My Climb Log Aug25'!$M$58:$M$65</definedName>
-    <definedName name="_xlchart.v2.20" hidden="1">'My ClimbRecov24_25'!$B$81:$B$88</definedName>
-    <definedName name="_xlchart.v2.21" hidden="1">'My ClimbRecov24_25'!$C$80</definedName>
-    <definedName name="_xlchart.v2.22" hidden="1">'My ClimbRecov24_25'!$C$81:$C$88</definedName>
-    <definedName name="_xlchart.v2.23" hidden="1">'My ClimbRecov24_25'!$L$32:$L$39</definedName>
-    <definedName name="_xlchart.v2.24" hidden="1">'My ClimbRecov24_25'!$N$32:$N$39</definedName>
-    <definedName name="_xlchart.v2.25" hidden="1">'My ClimbRecov24_25'!$L$158:$L$165</definedName>
-    <definedName name="_xlchart.v2.26" hidden="1">'My ClimbRecov24_25'!$N$157</definedName>
-    <definedName name="_xlchart.v2.27" hidden="1">'My ClimbRecov24_25'!$N$158:$N$165</definedName>
-    <definedName name="_xlchart.v2.28" hidden="1">'My ClimbRecov24_25'!$L$88:$L$95</definedName>
-    <definedName name="_xlchart.v2.29" hidden="1">'My ClimbRecov24_25'!$M$87</definedName>
+    <definedName name="_xlchart.v2.1" hidden="1">'My Climb Log Aug25'!$N$57</definedName>
+    <definedName name="_xlchart.v2.10" hidden="1">'My ClimbRecov24_25'!$N$302:$N$309</definedName>
+    <definedName name="_xlchart.v2.11" hidden="1">'My ClimbRecov24_25'!$L$230:$L$237</definedName>
+    <definedName name="_xlchart.v2.12" hidden="1">'My ClimbRecov24_25'!$M$229</definedName>
+    <definedName name="_xlchart.v2.13" hidden="1">'My ClimbRecov24_25'!$M$230:$M$237</definedName>
+    <definedName name="_xlchart.v2.14" hidden="1">'My ClimbRecov24_25'!$L$88:$L$95</definedName>
+    <definedName name="_xlchart.v2.15" hidden="1">'My ClimbRecov24_25'!$M$87</definedName>
+    <definedName name="_xlchart.v2.16" hidden="1">'My ClimbRecov24_25'!$M$88:$M$95</definedName>
+    <definedName name="_xlchart.v2.17" hidden="1">'My ClimbRecov24_25'!$L$158:$L$165</definedName>
+    <definedName name="_xlchart.v2.18" hidden="1">'My ClimbRecov24_25'!$M$157</definedName>
+    <definedName name="_xlchart.v2.19" hidden="1">'My ClimbRecov24_25'!$M$158:$M$165</definedName>
+    <definedName name="_xlchart.v2.2" hidden="1">'My Climb Log Aug25'!$N$58:$N$65</definedName>
+    <definedName name="_xlchart.v2.20" hidden="1">'My ClimbRecov24_25'!$L$32:$L$39</definedName>
+    <definedName name="_xlchart.v2.21" hidden="1">'My ClimbRecov24_25'!$M$31</definedName>
+    <definedName name="_xlchart.v2.22" hidden="1">'My ClimbRecov24_25'!$M$32:$M$39</definedName>
+    <definedName name="_xlchart.v2.23" hidden="1">'My ClimbRecov24_25'!$L$302:$L$309</definedName>
+    <definedName name="_xlchart.v2.24" hidden="1">'My ClimbRecov24_25'!$N$301</definedName>
+    <definedName name="_xlchart.v2.25" hidden="1">'My ClimbRecov24_25'!$N$302:$N$309</definedName>
+    <definedName name="_xlchart.v2.26" hidden="1">'My ClimbRecov24_25'!$B$81:$B$88</definedName>
+    <definedName name="_xlchart.v2.27" hidden="1">'My ClimbRecov24_25'!$C$80</definedName>
+    <definedName name="_xlchart.v2.28" hidden="1">'My ClimbRecov24_25'!$C$81:$C$88</definedName>
+    <definedName name="_xlchart.v2.29" hidden="1">'My ClimbRecov24_25'!$L$230:$L$237</definedName>
     <definedName name="_xlchart.v2.3" hidden="1">'My Climb Log Aug25'!$L$58:$L$65</definedName>
-    <definedName name="_xlchart.v2.30" hidden="1">'My ClimbRecov24_25'!$M$88:$M$95</definedName>
-    <definedName name="_xlchart.v2.31" hidden="1">'My ClimbRecov24_25'!$L$158:$L$165</definedName>
-    <definedName name="_xlchart.v2.32" hidden="1">'My ClimbRecov24_25'!$M$157</definedName>
-    <definedName name="_xlchart.v2.33" hidden="1">'My ClimbRecov24_25'!$M$158:$M$165</definedName>
-    <definedName name="_xlchart.v2.34" hidden="1">'My ClimbRecov24_25'!$L$32:$L$39</definedName>
-    <definedName name="_xlchart.v2.35" hidden="1">'My ClimbRecov24_25'!$M$31</definedName>
-    <definedName name="_xlchart.v2.36" hidden="1">'My ClimbRecov24_25'!$M$32:$M$39</definedName>
-    <definedName name="_xlchart.v2.37" hidden="1">'My ClimbRecov24_25'!$L$230:$L$237</definedName>
-    <definedName name="_xlchart.v2.38" hidden="1">'My ClimbRecov24_25'!$N$229</definedName>
-    <definedName name="_xlchart.v2.39" hidden="1">'My ClimbRecov24_25'!$N$230:$N$237</definedName>
-    <definedName name="_xlchart.v2.4" hidden="1">'My Climb Log Aug25'!$N$57</definedName>
-    <definedName name="_xlchart.v2.40" hidden="1">'My ClimbRecov24_25'!$L$302:$L$309</definedName>
-    <definedName name="_xlchart.v2.41" hidden="1">'My ClimbRecov24_25'!$N$301</definedName>
-    <definedName name="_xlchart.v2.42" hidden="1">'My ClimbRecov24_25'!$N$302:$N$309</definedName>
-    <definedName name="_xlchart.v2.43" hidden="1">'My ClimbRecov24_25'!$L$302:$L$309</definedName>
-    <definedName name="_xlchart.v2.44" hidden="1">'My ClimbRecov24_25'!$M$302:$M$309</definedName>
-    <definedName name="_xlchart.v2.5" hidden="1">'My Climb Log Aug25'!$N$58:$N$65</definedName>
-    <definedName name="_xlchart.v2.6" hidden="1">'My ClimbRecov24_25'!$B$81:$B$88</definedName>
-    <definedName name="_xlchart.v2.7" hidden="1">'My ClimbRecov24_25'!$D$80</definedName>
-    <definedName name="_xlchart.v2.8" hidden="1">'My ClimbRecov24_25'!$D$81:$D$88</definedName>
-    <definedName name="_xlchart.v2.9" hidden="1">'My ClimbRecov24_25'!$L$230:$L$237</definedName>
+    <definedName name="_xlchart.v2.30" hidden="1">'My ClimbRecov24_25'!$N$229</definedName>
+    <definedName name="_xlchart.v2.31" hidden="1">'My ClimbRecov24_25'!$N$230:$N$237</definedName>
+    <definedName name="_xlchart.v2.32" hidden="1">'My ClimbRecov24_25'!$L$302:$L$309</definedName>
+    <definedName name="_xlchart.v2.33" hidden="1">'My ClimbRecov24_25'!$M$302:$M$309</definedName>
+    <definedName name="_xlchart.v2.34" hidden="1">'My ClimbRecov24_25'!$L$158:$L$165</definedName>
+    <definedName name="_xlchart.v2.35" hidden="1">'My ClimbRecov24_25'!$N$157</definedName>
+    <definedName name="_xlchart.v2.36" hidden="1">'My ClimbRecov24_25'!$N$158:$N$165</definedName>
+    <definedName name="_xlchart.v2.37" hidden="1">'My ClimbRecov24_25'!$L$32:$L$39</definedName>
+    <definedName name="_xlchart.v2.38" hidden="1">'My ClimbRecov24_25'!$N$32:$N$39</definedName>
+    <definedName name="_xlchart.v2.39" hidden="1">'My ClimbRecov24_25'!$B$81:$B$88</definedName>
+    <definedName name="_xlchart.v2.4" hidden="1">'My Climb Log Aug25'!$M$57</definedName>
+    <definedName name="_xlchart.v2.40" hidden="1">'My ClimbRecov24_25'!$D$80</definedName>
+    <definedName name="_xlchart.v2.41" hidden="1">'My ClimbRecov24_25'!$D$81:$D$88</definedName>
+    <definedName name="_xlchart.v2.42" hidden="1">'My ClimbRecov24_25'!$L$88:$L$95</definedName>
+    <definedName name="_xlchart.v2.43" hidden="1">'My ClimbRecov24_25'!$N$87</definedName>
+    <definedName name="_xlchart.v2.44" hidden="1">'My ClimbRecov24_25'!$N$88:$N$95</definedName>
+    <definedName name="_xlchart.v2.5" hidden="1">'My Climb Log Aug25'!$M$58:$M$65</definedName>
+    <definedName name="_xlchart.v2.6" hidden="1">'My ClimbRecov24_25'!$L$302:$L$309</definedName>
+    <definedName name="_xlchart.v2.7" hidden="1">'My ClimbRecov24_25'!$M$302:$M$309</definedName>
+    <definedName name="_xlchart.v2.8" hidden="1">'My ClimbRecov24_25'!$L$302:$L$309</definedName>
+    <definedName name="_xlchart.v2.9" hidden="1">'My ClimbRecov24_25'!$N$301</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1299,7 +1299,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4665" uniqueCount="485">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4828" uniqueCount="486">
   <si>
     <t>Training Gym 2024</t>
   </si>
@@ -2859,6 +2859,9 @@
   </si>
   <si>
     <t>forgot and added 2.5kg</t>
+  </si>
+  <si>
+    <t>Small wooden ball</t>
   </si>
 </sst>
 </file>
@@ -4860,6 +4863,45 @@
     <xf numFmtId="164" fontId="0" fillId="24" borderId="31" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="24" borderId="44" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="46" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="17" fontId="20" fillId="31" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="22" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="35" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="20" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="28" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
@@ -4868,9 +4910,6 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="28" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="23" borderId="57" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -4926,13 +4965,61 @@
     <xf numFmtId="0" fontId="0" fillId="17" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="47" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="58" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="68" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="60" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="60" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="61" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="59" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
@@ -4941,13 +5028,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="59" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4959,90 +5046,6 @@
     <xf numFmtId="0" fontId="0" fillId="15" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="60" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="61" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="60" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="68" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="47" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="58" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="17" fontId="20" fillId="31" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="9" fontId="22" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="35" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="20" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -8745,10 +8748,10 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:strDim type="cat">
-        <cx:f>_xlchart.v2.0</cx:f>
+        <cx:f>_xlchart.v2.3</cx:f>
       </cx:strDim>
       <cx:numDim type="val">
-        <cx:f>_xlchart.v2.2</cx:f>
+        <cx:f>_xlchart.v2.5</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -8786,7 +8789,7 @@
         <cx:series layoutId="funnel" uniqueId="{A003F98F-E273-486D-B8EF-26A149080445}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v2.1</cx:f>
+              <cx:f>_xlchart.v2.4</cx:f>
               <cx:v>nr.Rotes</cx:v>
             </cx:txData>
           </cx:tx>
@@ -8810,10 +8813,10 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:strDim type="cat">
-        <cx:f>_xlchart.v2.6</cx:f>
+        <cx:f>_xlchart.v2.39</cx:f>
       </cx:strDim>
       <cx:numDim type="val">
-        <cx:f>_xlchart.v2.8</cx:f>
+        <cx:f>_xlchart.v2.41</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -8851,7 +8854,7 @@
         <cx:series layoutId="funnel" uniqueId="{30CD089F-9800-4F70-AE9C-3640537393FD}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v2.7</cx:f>
+              <cx:f>_xlchart.v2.40</cx:f>
               <cx:v>m/grade</cx:v>
             </cx:txData>
           </cx:tx>
@@ -8883,10 +8886,10 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:strDim type="cat">
-        <cx:f>_xlchart.v2.9</cx:f>
+        <cx:f>_xlchart.v2.11</cx:f>
       </cx:strDim>
       <cx:numDim type="val">
-        <cx:f>_xlchart.v2.11</cx:f>
+        <cx:f>_xlchart.v2.13</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -8924,7 +8927,7 @@
         <cx:series layoutId="funnel" uniqueId="{FB8DBC82-27A8-4406-AC11-A1B1077C2F7E}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v2.10</cx:f>
+              <cx:f>_xlchart.v2.12</cx:f>
               <cx:v>nr.Rotes</cx:v>
             </cx:txData>
           </cx:tx>
@@ -8948,10 +8951,10 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:strDim type="cat">
-        <cx:f>_xlchart.v2.37</cx:f>
+        <cx:f>_xlchart.v2.29</cx:f>
       </cx:strDim>
       <cx:numDim type="val">
-        <cx:f>_xlchart.v2.39</cx:f>
+        <cx:f>_xlchart.v2.31</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -8989,7 +8992,7 @@
         <cx:series layoutId="funnel" uniqueId="{C19CD63B-CB55-4793-9446-CAAF56F211D3}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v2.38</cx:f>
+              <cx:f>_xlchart.v2.30</cx:f>
               <cx:v>m/grade</cx:v>
             </cx:txData>
           </cx:tx>
@@ -9013,10 +9016,10 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:strDim type="cat">
-        <cx:f>_xlchart.v2.15</cx:f>
+        <cx:f>_xlchart.v2.32</cx:f>
       </cx:strDim>
       <cx:numDim type="val">
-        <cx:f>_xlchart.v2.16</cx:f>
+        <cx:f>_xlchart.v2.33</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -9072,10 +9075,10 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:strDim type="cat">
-        <cx:f>_xlchart.v2.12</cx:f>
+        <cx:f>_xlchart.v2.8</cx:f>
       </cx:strDim>
       <cx:numDim type="val">
-        <cx:f>_xlchart.v2.14</cx:f>
+        <cx:f>_xlchart.v2.10</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -9113,7 +9116,7 @@
         <cx:series layoutId="funnel" uniqueId="{73B27DE1-6057-440E-AE7A-4EAB15428715}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v2.13</cx:f>
+              <cx:f>_xlchart.v2.9</cx:f>
               <cx:v>m/grade</cx:v>
             </cx:txData>
           </cx:tx>
@@ -9137,10 +9140,10 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:strDim type="cat">
-        <cx:f>_xlchart.v2.43</cx:f>
+        <cx:f>_xlchart.v2.6</cx:f>
       </cx:strDim>
       <cx:numDim type="val">
-        <cx:f>_xlchart.v2.44</cx:f>
+        <cx:f>_xlchart.v2.7</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -9196,10 +9199,10 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:strDim type="cat">
-        <cx:f>_xlchart.v2.40</cx:f>
+        <cx:f>_xlchart.v2.23</cx:f>
       </cx:strDim>
       <cx:numDim type="val">
-        <cx:f>_xlchart.v2.42</cx:f>
+        <cx:f>_xlchart.v2.25</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -9237,7 +9240,7 @@
         <cx:series layoutId="funnel" uniqueId="{73B27DE1-6057-440E-AE7A-4EAB15428715}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v2.41</cx:f>
+              <cx:f>_xlchart.v2.24</cx:f>
               <cx:v>m/grade</cx:v>
             </cx:txData>
           </cx:tx>
@@ -9261,10 +9264,10 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:strDim type="cat">
-        <cx:f>_xlchart.v2.3</cx:f>
+        <cx:f>_xlchart.v2.0</cx:f>
       </cx:strDim>
       <cx:numDim type="val">
-        <cx:f>_xlchart.v2.5</cx:f>
+        <cx:f>_xlchart.v2.2</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -9302,7 +9305,7 @@
         <cx:series layoutId="funnel" uniqueId="{A4ED4C9B-2694-4B9B-A798-8D85DE668EBF}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v2.4</cx:f>
+              <cx:f>_xlchart.v2.1</cx:f>
               <cx:v>m/grade</cx:v>
             </cx:txData>
           </cx:tx>
@@ -9326,10 +9329,10 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:strDim type="cat">
-        <cx:f>_xlchart.v2.34</cx:f>
+        <cx:f>_xlchart.v2.20</cx:f>
       </cx:strDim>
       <cx:numDim type="val">
-        <cx:f>_xlchart.v2.36</cx:f>
+        <cx:f>_xlchart.v2.22</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -9367,7 +9370,7 @@
         <cx:series layoutId="funnel" uniqueId="{EFCC1542-F3B6-43DF-8633-A1BFE57A93E8}" formatIdx="0">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v2.35</cx:f>
+              <cx:f>_xlchart.v2.21</cx:f>
               <cx:v>nr.Rotes</cx:v>
             </cx:txData>
           </cx:tx>
@@ -9398,10 +9401,10 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:strDim type="cat">
-        <cx:f>_xlchart.v2.23</cx:f>
+        <cx:f>_xlchart.v2.37</cx:f>
       </cx:strDim>
       <cx:numDim type="val">
-        <cx:f>_xlchart.v2.24</cx:f>
+        <cx:f>_xlchart.v2.38</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -9457,10 +9460,10 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:strDim type="cat">
-        <cx:f>_xlchart.v2.17</cx:f>
+        <cx:f>_xlchart.v2.42</cx:f>
       </cx:strDim>
       <cx:numDim type="val">
-        <cx:f>_xlchart.v2.19</cx:f>
+        <cx:f>_xlchart.v2.44</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -9514,7 +9517,7 @@
         <cx:series layoutId="funnel" uniqueId="{B4D0ECFE-ABDC-4262-BAE3-93968816F03F}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v2.18</cx:f>
+              <cx:f>_xlchart.v2.43</cx:f>
               <cx:v>m/grade</cx:v>
             </cx:txData>
           </cx:tx>
@@ -9535,10 +9538,10 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:strDim type="cat">
-        <cx:f>_xlchart.v2.28</cx:f>
+        <cx:f>_xlchart.v2.14</cx:f>
       </cx:strDim>
       <cx:numDim type="val">
-        <cx:f>_xlchart.v2.30</cx:f>
+        <cx:f>_xlchart.v2.16</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -9590,7 +9593,7 @@
         <cx:series layoutId="funnel" uniqueId="{05C44B17-8238-4100-B6E8-1D53ECC2B072}" formatIdx="0">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v2.29</cx:f>
+              <cx:f>_xlchart.v2.15</cx:f>
               <cx:v>nr.Rotes</cx:v>
             </cx:txData>
           </cx:tx>
@@ -9611,10 +9614,10 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:strDim type="cat">
-        <cx:f>_xlchart.v2.31</cx:f>
+        <cx:f>_xlchart.v2.17</cx:f>
       </cx:strDim>
       <cx:numDim type="val">
-        <cx:f>_xlchart.v2.33</cx:f>
+        <cx:f>_xlchart.v2.19</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -9652,7 +9655,7 @@
         <cx:series layoutId="funnel" uniqueId="{2447EB50-6D72-4713-AA9A-F22BBD682711}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v2.32</cx:f>
+              <cx:f>_xlchart.v2.18</cx:f>
               <cx:v>nr.Rotes</cx:v>
             </cx:txData>
           </cx:tx>
@@ -9676,10 +9679,10 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:strDim type="cat">
-        <cx:f>_xlchart.v2.25</cx:f>
+        <cx:f>_xlchart.v2.34</cx:f>
       </cx:strDim>
       <cx:numDim type="val">
-        <cx:f>_xlchart.v2.27</cx:f>
+        <cx:f>_xlchart.v2.36</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -9717,7 +9720,7 @@
         <cx:series layoutId="funnel" uniqueId="{702D742B-6ED9-4147-9E5B-C7D526EF3646}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v2.26</cx:f>
+              <cx:f>_xlchart.v2.35</cx:f>
               <cx:v>m/grade</cx:v>
             </cx:txData>
           </cx:tx>
@@ -9741,10 +9744,10 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:strDim type="cat">
-        <cx:f>_xlchart.v2.20</cx:f>
+        <cx:f>_xlchart.v2.26</cx:f>
       </cx:strDim>
       <cx:numDim type="val">
-        <cx:f>_xlchart.v2.22</cx:f>
+        <cx:f>_xlchart.v2.28</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -9782,7 +9785,7 @@
         <cx:series layoutId="funnel" uniqueId="{A7BD6AF6-3C17-4CEB-8A87-10A5DA0CFF47}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v2.21</cx:f>
+              <cx:f>_xlchart.v2.27</cx:f>
               <cx:v>nr.Rotes</cx:v>
             </cx:txData>
           </cx:tx>
@@ -24575,10 +24578,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -26340,17 +26339,17 @@
       <c r="I56" s="5"/>
     </row>
     <row r="59" spans="2:15" x14ac:dyDescent="0.2">
-      <c r="C59" s="333" t="s">
+      <c r="C59" s="352" t="s">
         <v>455</v>
       </c>
-      <c r="D59" s="333"/>
-      <c r="E59" s="333"/>
-      <c r="F59" s="333"/>
-      <c r="G59" s="333"/>
-      <c r="H59" s="333"/>
-      <c r="I59" s="333"/>
-      <c r="J59" s="333"/>
-      <c r="K59" s="333"/>
+      <c r="D59" s="352"/>
+      <c r="E59" s="352"/>
+      <c r="F59" s="352"/>
+      <c r="G59" s="352"/>
+      <c r="H59" s="352"/>
+      <c r="I59" s="352"/>
+      <c r="J59" s="352"/>
+      <c r="K59" s="352"/>
       <c r="M59" s="15" t="s">
         <v>431</v>
       </c>
@@ -38483,7 +38482,7 @@
     <row r="169" spans="35:64" ht="14.5" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="172" spans="35:64" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="173" spans="35:64" x14ac:dyDescent="0.2">
-      <c r="AI173" s="330" t="s">
+      <c r="AI173" s="353" t="s">
         <v>228</v>
       </c>
       <c r="AJ173" s="142" t="s">
@@ -38519,7 +38518,7 @@
       <c r="AT173" s="51" t="s">
         <v>222</v>
       </c>
-      <c r="BA173" s="330" t="s">
+      <c r="BA173" s="353" t="s">
         <v>228</v>
       </c>
       <c r="BB173" s="142" t="s">
@@ -38557,7 +38556,7 @@
       </c>
     </row>
     <row r="174" spans="35:64" x14ac:dyDescent="0.2">
-      <c r="AI174" s="331"/>
+      <c r="AI174" s="354"/>
       <c r="AJ174" s="39" t="s">
         <v>227</v>
       </c>
@@ -38591,7 +38590,7 @@
       <c r="AT174" s="54" t="s">
         <v>223</v>
       </c>
-      <c r="BA174" s="331"/>
+      <c r="BA174" s="354"/>
       <c r="BB174" s="39" t="s">
         <v>227</v>
       </c>
@@ -38627,13 +38626,13 @@
       </c>
     </row>
     <row r="175" spans="35:64" x14ac:dyDescent="0.2">
-      <c r="AI175" s="331"/>
+      <c r="AI175" s="354"/>
       <c r="AT175" s="146"/>
-      <c r="BA175" s="331"/>
+      <c r="BA175" s="354"/>
       <c r="BL175" s="146"/>
     </row>
     <row r="176" spans="35:64" x14ac:dyDescent="0.2">
-      <c r="AI176" s="331"/>
+      <c r="AI176" s="354"/>
       <c r="AJ176" s="127" t="s">
         <v>221</v>
       </c>
@@ -38667,7 +38666,7 @@
       <c r="AT176" s="54" t="s">
         <v>222</v>
       </c>
-      <c r="BA176" s="331"/>
+      <c r="BA176" s="354"/>
       <c r="BB176" s="127" t="s">
         <v>221</v>
       </c>
@@ -38703,7 +38702,7 @@
       </c>
     </row>
     <row r="177" spans="35:64" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="AI177" s="332"/>
+      <c r="AI177" s="355"/>
       <c r="AJ177" s="147" t="s">
         <v>226</v>
       </c>
@@ -38737,7 +38736,7 @@
       <c r="AT177" s="43" t="s">
         <v>229</v>
       </c>
-      <c r="BA177" s="332"/>
+      <c r="BA177" s="355"/>
       <c r="BB177" s="147" t="s">
         <v>226</v>
       </c>
@@ -39482,596 +39481,599 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD74C1BA-CEDA-A443-A105-A99351A4C8B6}">
-  <dimension ref="A2:Q24"/>
+  <dimension ref="A2:Q60"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="24.5" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="2" spans="1:17" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="379"/>
-      <c r="B2" s="379"/>
-      <c r="C2" s="379"/>
-      <c r="D2" s="379"/>
-      <c r="E2" s="379"/>
-      <c r="F2" s="379"/>
-      <c r="G2" s="379"/>
-      <c r="H2" s="379"/>
-      <c r="I2" s="379"/>
-      <c r="J2" s="379"/>
-      <c r="K2" s="379"/>
-      <c r="L2" s="379"/>
-      <c r="M2" s="379"/>
-      <c r="N2" s="379"/>
-      <c r="O2" s="379"/>
-      <c r="P2" s="379"/>
-      <c r="Q2" s="379"/>
+      <c r="A2" s="330"/>
+      <c r="B2" s="330"/>
+      <c r="C2" s="330"/>
+      <c r="D2" s="330"/>
+      <c r="E2" s="330"/>
+      <c r="F2" s="330"/>
+      <c r="G2" s="330"/>
+      <c r="H2" s="330"/>
+      <c r="I2" s="330"/>
+      <c r="J2" s="330"/>
+      <c r="K2" s="330"/>
+      <c r="L2" s="330"/>
+      <c r="M2" s="330"/>
+      <c r="N2" s="330"/>
+      <c r="O2" s="330"/>
+      <c r="P2" s="330"/>
+      <c r="Q2" s="330"/>
     </row>
     <row r="3" spans="1:17" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="379"/>
-      <c r="B3" s="379"/>
-      <c r="C3" s="380" t="s">
+      <c r="A3" s="330"/>
+      <c r="B3" s="330"/>
+      <c r="C3" s="331" t="s">
         <v>261</v>
       </c>
-      <c r="D3" s="381"/>
-      <c r="E3" s="381"/>
-      <c r="F3" s="382"/>
-      <c r="G3" s="382"/>
-      <c r="H3" s="382"/>
-      <c r="I3" s="383"/>
-      <c r="J3" s="383"/>
-      <c r="K3" s="384">
+      <c r="D3" s="332"/>
+      <c r="E3" s="332"/>
+      <c r="F3" s="333"/>
+      <c r="G3" s="333"/>
+      <c r="H3" s="333"/>
+      <c r="I3" s="334"/>
+      <c r="J3" s="334"/>
+      <c r="K3" s="335">
         <v>46205</v>
       </c>
-      <c r="L3" s="379"/>
-      <c r="M3" s="379"/>
-      <c r="N3" s="379"/>
-      <c r="O3" s="379"/>
-      <c r="P3" s="379"/>
-      <c r="Q3" s="379"/>
+      <c r="L3" s="330"/>
+      <c r="M3" s="330"/>
+      <c r="N3" s="330"/>
+      <c r="O3" s="330"/>
+      <c r="P3" s="330"/>
+      <c r="Q3" s="330"/>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A4" s="379"/>
-      <c r="B4" s="379">
+      <c r="A4" s="330"/>
+      <c r="B4" s="330">
         <v>1</v>
       </c>
-      <c r="C4" s="379" t="s">
+      <c r="C4" s="330" t="s">
         <v>262</v>
       </c>
-      <c r="D4" s="379"/>
-      <c r="E4" s="385"/>
-      <c r="F4" s="385"/>
-      <c r="G4" s="385"/>
-      <c r="H4" s="385"/>
-      <c r="I4" s="379"/>
-      <c r="J4" s="379"/>
-      <c r="K4" s="386">
+      <c r="D4" s="330"/>
+      <c r="E4" s="336"/>
+      <c r="F4" s="336"/>
+      <c r="G4" s="336"/>
+      <c r="H4" s="336"/>
+      <c r="I4" s="330"/>
+      <c r="J4" s="330"/>
+      <c r="K4" s="337">
         <v>51.5</v>
       </c>
-      <c r="L4" s="379" t="s">
+      <c r="L4" s="330" t="s">
         <v>479</v>
       </c>
-      <c r="M4" s="379"/>
-      <c r="N4" s="379"/>
-      <c r="O4" s="379"/>
-      <c r="P4" s="379"/>
-      <c r="Q4" s="379"/>
+      <c r="M4" s="330"/>
+      <c r="N4" s="330"/>
+      <c r="O4" s="330"/>
+      <c r="P4" s="330"/>
+      <c r="Q4" s="330"/>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A5" s="379"/>
-      <c r="B5" s="379">
+      <c r="A5" s="330"/>
+      <c r="B5" s="330">
         <v>2</v>
       </c>
-      <c r="C5" s="379" t="s">
+      <c r="C5" s="330" t="s">
         <v>264</v>
       </c>
-      <c r="D5" s="379"/>
-      <c r="E5" s="385"/>
-      <c r="F5" s="385"/>
-      <c r="G5" s="385"/>
-      <c r="H5" s="385"/>
-      <c r="I5" s="379"/>
-      <c r="J5" s="379"/>
-      <c r="K5" s="386" t="s">
+      <c r="D5" s="330"/>
+      <c r="E5" s="336"/>
+      <c r="F5" s="336"/>
+      <c r="G5" s="336"/>
+      <c r="H5" s="336"/>
+      <c r="I5" s="330"/>
+      <c r="J5" s="330"/>
+      <c r="K5" s="337" t="s">
         <v>265</v>
       </c>
-      <c r="L5" s="379" t="s">
+      <c r="L5" s="330" t="s">
         <v>480</v>
       </c>
-      <c r="M5" s="379"/>
-      <c r="N5" s="379"/>
-      <c r="O5" s="379"/>
-      <c r="P5" s="379"/>
-      <c r="Q5" s="379"/>
+      <c r="M5" s="330"/>
+      <c r="N5" s="330"/>
+      <c r="O5" s="330"/>
+      <c r="P5" s="330"/>
+      <c r="Q5" s="330"/>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A6" s="379"/>
-      <c r="B6" s="379">
+      <c r="A6" s="330"/>
+      <c r="B6" s="330">
         <v>3</v>
       </c>
-      <c r="C6" s="379" t="s">
+      <c r="C6" s="330" t="s">
         <v>266</v>
       </c>
-      <c r="D6" s="379"/>
-      <c r="E6" s="385"/>
-      <c r="F6" s="385"/>
-      <c r="G6" s="385"/>
-      <c r="H6" s="385"/>
-      <c r="I6" s="379"/>
-      <c r="J6" s="379"/>
-      <c r="K6" s="385" t="s">
+      <c r="D6" s="330"/>
+      <c r="E6" s="336"/>
+      <c r="F6" s="336"/>
+      <c r="G6" s="336"/>
+      <c r="H6" s="336"/>
+      <c r="I6" s="330"/>
+      <c r="J6" s="330"/>
+      <c r="K6" s="336" t="s">
         <v>482</v>
       </c>
-      <c r="L6" s="379" t="s">
+      <c r="L6" s="330" t="s">
         <v>481</v>
       </c>
-      <c r="M6" s="379"/>
-      <c r="N6" s="379"/>
-      <c r="O6" s="379"/>
-      <c r="P6" s="379"/>
-      <c r="Q6" s="379"/>
+      <c r="M6" s="330"/>
+      <c r="N6" s="330"/>
+      <c r="O6" s="330"/>
+      <c r="P6" s="330"/>
+      <c r="Q6" s="330"/>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A7" s="379"/>
-      <c r="B7" s="379">
+      <c r="A7" s="330"/>
+      <c r="B7" s="330">
         <v>4</v>
       </c>
-      <c r="C7" s="379" t="s">
+      <c r="C7" s="330" t="s">
         <v>268</v>
       </c>
-      <c r="D7" s="379"/>
-      <c r="E7" s="386" t="s">
+      <c r="D7" s="330"/>
+      <c r="E7" s="337" t="s">
         <v>273</v>
       </c>
-      <c r="F7" s="386"/>
-      <c r="G7" s="385"/>
-      <c r="H7" s="385"/>
-      <c r="I7" s="379" t="s">
+      <c r="F7" s="337"/>
+      <c r="G7" s="336"/>
+      <c r="H7" s="336"/>
+      <c r="I7" s="330" t="s">
         <v>275</v>
       </c>
-      <c r="J7" s="379"/>
-      <c r="K7" s="385">
+      <c r="J7" s="330"/>
+      <c r="K7" s="336">
         <v>30.5</v>
       </c>
-      <c r="L7" s="379"/>
-      <c r="M7" s="379"/>
-      <c r="N7" s="379"/>
-      <c r="O7" s="379"/>
-      <c r="P7" s="379"/>
-      <c r="Q7" s="379"/>
+      <c r="L7" s="330"/>
+      <c r="M7" s="330"/>
+      <c r="N7" s="330"/>
+      <c r="O7" s="330"/>
+      <c r="P7" s="330"/>
+      <c r="Q7" s="330"/>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A8" s="379"/>
-      <c r="B8" s="379">
+      <c r="A8" s="330"/>
+      <c r="B8" s="330">
         <v>5</v>
       </c>
-      <c r="C8" s="379" t="s">
+      <c r="C8" s="330" t="s">
         <v>270</v>
       </c>
-      <c r="D8" s="385"/>
-      <c r="E8" s="386" t="s">
+      <c r="D8" s="336"/>
+      <c r="E8" s="337" t="s">
         <v>274</v>
       </c>
-      <c r="F8" s="386"/>
-      <c r="G8" s="386"/>
-      <c r="H8" s="385">
+      <c r="F8" s="337"/>
+      <c r="G8" s="337"/>
+      <c r="H8" s="336">
         <v>2.5</v>
       </c>
-      <c r="I8" s="379" t="s">
+      <c r="I8" s="330" t="s">
         <v>275</v>
       </c>
-      <c r="J8" s="379"/>
-      <c r="K8" s="385" t="s">
+      <c r="J8" s="330"/>
+      <c r="K8" s="336" t="s">
         <v>483</v>
       </c>
-      <c r="L8" s="379" t="s">
+      <c r="L8" s="330" t="s">
         <v>484</v>
       </c>
-      <c r="M8" s="379"/>
-      <c r="N8" s="379"/>
-      <c r="O8" s="379"/>
-      <c r="P8" s="379"/>
-      <c r="Q8" s="379"/>
+      <c r="M8" s="330"/>
+      <c r="N8" s="330"/>
+      <c r="O8" s="330"/>
+      <c r="P8" s="330"/>
+      <c r="Q8" s="330"/>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A9" s="379"/>
-      <c r="B9" s="379"/>
-      <c r="C9" s="379"/>
-      <c r="D9" s="379"/>
-      <c r="E9" s="379"/>
-      <c r="F9" s="379"/>
-      <c r="G9" s="379"/>
-      <c r="H9" s="379"/>
-      <c r="I9" s="379"/>
-      <c r="J9" s="379"/>
-      <c r="K9" s="379"/>
-      <c r="L9" s="379"/>
-      <c r="M9" s="379"/>
-      <c r="N9" s="379"/>
-      <c r="O9" s="379"/>
-      <c r="P9" s="379"/>
-      <c r="Q9" s="379"/>
+      <c r="A9" s="330"/>
+      <c r="B9" s="330"/>
+      <c r="C9" s="330"/>
+      <c r="D9" s="330"/>
+      <c r="E9" s="330"/>
+      <c r="F9" s="330"/>
+      <c r="G9" s="330"/>
+      <c r="H9" s="330"/>
+      <c r="I9" s="330"/>
+      <c r="J9" s="330"/>
+      <c r="K9" s="330"/>
+      <c r="L9" s="330"/>
+      <c r="M9" s="330"/>
+      <c r="N9" s="330"/>
+      <c r="O9" s="330"/>
+      <c r="P9" s="330"/>
+      <c r="Q9" s="330"/>
     </row>
     <row r="10" spans="1:17" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="379"/>
-      <c r="B10" s="379"/>
-      <c r="C10" s="379"/>
-      <c r="D10" s="379"/>
-      <c r="E10" s="379"/>
-      <c r="F10" s="379"/>
-      <c r="G10" s="379"/>
-      <c r="H10" s="379"/>
-      <c r="I10" s="379"/>
-      <c r="J10" s="379"/>
-      <c r="K10" s="379"/>
-      <c r="L10" s="379"/>
-      <c r="M10" s="379"/>
-      <c r="N10" s="379"/>
-      <c r="O10" s="379"/>
-      <c r="P10" s="379"/>
-      <c r="Q10" s="379"/>
+      <c r="A10" s="330"/>
+      <c r="B10" s="330"/>
+      <c r="C10" s="330"/>
+      <c r="D10" s="330"/>
+      <c r="E10" s="330"/>
+      <c r="F10" s="330"/>
+      <c r="G10" s="330"/>
+      <c r="H10" s="330"/>
+      <c r="I10" s="330"/>
+      <c r="J10" s="330"/>
+      <c r="K10" s="330"/>
+      <c r="L10" s="330"/>
+      <c r="M10" s="330"/>
+      <c r="N10" s="330"/>
+      <c r="O10" s="330"/>
+      <c r="P10" s="330"/>
+      <c r="Q10" s="330"/>
     </row>
     <row r="11" spans="1:17" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="379"/>
-      <c r="B11" s="387" t="s">
+      <c r="A11" s="330"/>
+      <c r="B11" s="338" t="s">
         <v>386</v>
       </c>
-      <c r="C11" s="381" t="s">
+      <c r="C11" s="332" t="s">
         <v>261</v>
       </c>
-      <c r="D11" s="381"/>
-      <c r="E11" s="381"/>
-      <c r="F11" s="382"/>
-      <c r="G11" s="382"/>
-      <c r="H11" s="382"/>
-      <c r="I11" s="383"/>
-      <c r="J11" s="383"/>
-      <c r="K11" s="384">
+      <c r="D11" s="332"/>
+      <c r="E11" s="332"/>
+      <c r="F11" s="333"/>
+      <c r="G11" s="333"/>
+      <c r="H11" s="333"/>
+      <c r="I11" s="334"/>
+      <c r="J11" s="334"/>
+      <c r="K11" s="335">
         <v>46106</v>
       </c>
-      <c r="L11" s="379"/>
-      <c r="M11" s="379"/>
-      <c r="N11" s="379"/>
-      <c r="O11" s="379"/>
-      <c r="P11" s="379"/>
-      <c r="Q11" s="379"/>
+      <c r="L11" s="330"/>
+      <c r="M11" s="330"/>
+      <c r="N11" s="330"/>
+      <c r="O11" s="330"/>
+      <c r="P11" s="330"/>
+      <c r="Q11" s="330"/>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A12" s="379"/>
-      <c r="B12" s="388">
+      <c r="A12" s="330"/>
+      <c r="B12" s="339">
         <v>1</v>
       </c>
-      <c r="C12" s="379" t="s">
+      <c r="C12" s="330" t="s">
         <v>262</v>
       </c>
-      <c r="D12" s="379"/>
-      <c r="E12" s="385"/>
-      <c r="F12" s="385"/>
-      <c r="G12" s="385"/>
-      <c r="H12" s="385"/>
-      <c r="I12" s="379"/>
-      <c r="J12" s="379"/>
+      <c r="D12" s="330"/>
+      <c r="E12" s="336"/>
+      <c r="F12" s="336"/>
+      <c r="G12" s="336"/>
+      <c r="H12" s="336"/>
+      <c r="I12" s="330"/>
+      <c r="J12" s="330"/>
       <c r="K12" s="229" t="s">
         <v>383</v>
       </c>
-      <c r="L12" s="379"/>
-      <c r="M12" s="379"/>
-      <c r="N12" s="379"/>
-      <c r="O12" s="379"/>
-      <c r="P12" s="379"/>
-      <c r="Q12" s="379"/>
+      <c r="L12" s="330"/>
+      <c r="M12" s="330"/>
+      <c r="N12" s="330"/>
+      <c r="O12" s="330"/>
+      <c r="P12" s="330"/>
+      <c r="Q12" s="330"/>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A13" s="379"/>
-      <c r="B13" s="388">
+      <c r="A13" s="330"/>
+      <c r="B13" s="339">
         <v>2</v>
       </c>
-      <c r="C13" s="379" t="s">
+      <c r="C13" s="330" t="s">
         <v>264</v>
       </c>
-      <c r="D13" s="379"/>
-      <c r="E13" s="385" t="s">
+      <c r="D13" s="330"/>
+      <c r="E13" s="336" t="s">
         <v>387</v>
       </c>
-      <c r="F13" s="385" t="s">
+      <c r="F13" s="336" t="s">
         <v>388</v>
       </c>
-      <c r="G13" s="385"/>
-      <c r="H13" s="385"/>
-      <c r="I13" s="379"/>
-      <c r="J13" s="379"/>
+      <c r="G13" s="336"/>
+      <c r="H13" s="336"/>
+      <c r="I13" s="330"/>
+      <c r="J13" s="330"/>
       <c r="K13" s="229" t="s">
         <v>389</v>
       </c>
-      <c r="L13" s="379"/>
-      <c r="M13" s="379"/>
-      <c r="N13" s="379"/>
-      <c r="O13" s="379"/>
-      <c r="P13" s="379"/>
-      <c r="Q13" s="379"/>
+      <c r="L13" s="330"/>
+      <c r="M13" s="330"/>
+      <c r="N13" s="330"/>
+      <c r="O13" s="330"/>
+      <c r="P13" s="330"/>
+      <c r="Q13" s="330"/>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A14" s="379"/>
-      <c r="B14" s="389">
+      <c r="A14" s="330"/>
+      <c r="B14" s="340">
         <v>3</v>
       </c>
-      <c r="C14" s="379" t="s">
+      <c r="C14" s="330" t="s">
         <v>266</v>
       </c>
-      <c r="D14" s="379"/>
-      <c r="E14" s="385"/>
-      <c r="F14" s="385"/>
-      <c r="G14" s="385"/>
-      <c r="H14" s="385"/>
-      <c r="I14" s="379"/>
-      <c r="J14" s="379"/>
+      <c r="D14" s="330"/>
+      <c r="E14" s="336"/>
+      <c r="F14" s="336"/>
+      <c r="G14" s="336"/>
+      <c r="H14" s="336"/>
+      <c r="I14" s="330"/>
+      <c r="J14" s="330"/>
       <c r="K14" s="230" t="s">
         <v>384</v>
       </c>
-      <c r="L14" s="390" t="s">
+      <c r="L14" s="341" t="s">
         <v>21</v>
       </c>
-      <c r="M14" s="391" t="s">
+      <c r="M14" s="342" t="s">
         <v>214</v>
       </c>
-      <c r="N14" s="392" t="s">
+      <c r="N14" s="343" t="s">
         <v>210</v>
       </c>
-      <c r="O14" s="379"/>
-      <c r="P14" s="379"/>
-      <c r="Q14" s="379"/>
+      <c r="O14" s="330"/>
+      <c r="P14" s="330"/>
+      <c r="Q14" s="330"/>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A15" s="379"/>
-      <c r="B15" s="393">
+      <c r="A15" s="330"/>
+      <c r="B15" s="344">
         <v>4</v>
       </c>
-      <c r="C15" s="379" t="s">
+      <c r="C15" s="330" t="s">
         <v>385</v>
       </c>
-      <c r="D15" s="379"/>
-      <c r="E15" s="386" t="s">
+      <c r="D15" s="330"/>
+      <c r="E15" s="337" t="s">
         <v>273</v>
       </c>
-      <c r="F15" s="386"/>
-      <c r="G15" s="385"/>
-      <c r="H15" s="385"/>
-      <c r="I15" s="379" t="s">
+      <c r="F15" s="337"/>
+      <c r="G15" s="336"/>
+      <c r="H15" s="336"/>
+      <c r="I15" s="330" t="s">
         <v>275</v>
       </c>
-      <c r="J15" s="379"/>
+      <c r="J15" s="330"/>
       <c r="K15" s="242" t="s">
         <v>382</v>
       </c>
-      <c r="L15" s="379">
+      <c r="L15" s="330">
         <v>0.95</v>
       </c>
-      <c r="M15" s="379">
+      <c r="M15" s="330">
         <v>41.5</v>
       </c>
-      <c r="N15" s="394">
+      <c r="N15" s="345">
         <v>7</v>
       </c>
-      <c r="O15" s="379"/>
-      <c r="P15" s="379"/>
-      <c r="Q15" s="379"/>
+      <c r="O15" s="330"/>
+      <c r="P15" s="330"/>
+      <c r="Q15" s="330"/>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A16" s="379"/>
-      <c r="B16" s="395">
+      <c r="A16" s="330"/>
+      <c r="B16" s="346">
         <v>5</v>
       </c>
-      <c r="C16" s="379" t="s">
+      <c r="C16" s="330" t="s">
         <v>270</v>
       </c>
-      <c r="D16" s="385"/>
-      <c r="E16" s="386" t="s">
+      <c r="D16" s="336"/>
+      <c r="E16" s="337" t="s">
         <v>274</v>
       </c>
-      <c r="F16" s="386"/>
-      <c r="G16" s="386"/>
-      <c r="H16" s="385" t="s">
+      <c r="F16" s="337"/>
+      <c r="G16" s="337"/>
+      <c r="H16" s="336" t="s">
         <v>271</v>
       </c>
-      <c r="I16" s="379" t="s">
+      <c r="I16" s="330" t="s">
         <v>275</v>
       </c>
-      <c r="J16" s="379"/>
+      <c r="J16" s="330"/>
       <c r="K16" s="244" t="s">
         <v>404</v>
       </c>
-      <c r="L16" s="396">
+      <c r="L16" s="347">
         <v>190</v>
       </c>
-      <c r="M16" s="397" t="s">
+      <c r="M16" s="348" t="s">
         <v>405</v>
       </c>
-      <c r="N16" s="398">
+      <c r="N16" s="349">
         <v>3.17</v>
       </c>
-      <c r="O16" s="399" t="s">
+      <c r="O16" s="350" t="s">
         <v>406</v>
       </c>
-      <c r="P16" s="379"/>
-      <c r="Q16" s="379"/>
+      <c r="P16" s="330"/>
+      <c r="Q16" s="330"/>
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A17" s="379"/>
-      <c r="B17" s="379"/>
-      <c r="C17" s="379"/>
-      <c r="D17" s="379"/>
-      <c r="E17" s="379"/>
-      <c r="F17" s="379"/>
-      <c r="G17" s="379"/>
-      <c r="H17" s="379"/>
-      <c r="I17" s="379"/>
-      <c r="J17" s="379"/>
-      <c r="K17" s="379"/>
-      <c r="L17" s="379"/>
-      <c r="M17" s="379"/>
-      <c r="N17" s="379"/>
-      <c r="O17" s="379"/>
-      <c r="P17" s="379"/>
-      <c r="Q17" s="379"/>
+      <c r="A17" s="330"/>
+      <c r="B17" s="330"/>
+      <c r="C17" s="330"/>
+      <c r="D17" s="330"/>
+      <c r="E17" s="330"/>
+      <c r="F17" s="330"/>
+      <c r="G17" s="330"/>
+      <c r="H17" s="330"/>
+      <c r="I17" s="330"/>
+      <c r="J17" s="330"/>
+      <c r="K17" s="330"/>
+      <c r="L17" s="330"/>
+      <c r="M17" s="330"/>
+      <c r="N17" s="330"/>
+      <c r="O17" s="330"/>
+      <c r="P17" s="330"/>
+      <c r="Q17" s="330"/>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A18" s="379"/>
-      <c r="B18" s="379" t="s">
+      <c r="A18" s="330"/>
+      <c r="B18" s="330" t="s">
         <v>393</v>
       </c>
-      <c r="C18" s="379" t="s">
+      <c r="C18" s="330" t="s">
         <v>396</v>
       </c>
-      <c r="D18" s="379"/>
-      <c r="E18" s="379"/>
-      <c r="F18" s="379"/>
-      <c r="G18" s="379"/>
-      <c r="H18" s="379"/>
-      <c r="I18" s="379"/>
-      <c r="J18" s="379"/>
-      <c r="K18" s="379"/>
-      <c r="L18" s="379"/>
-      <c r="M18" s="379"/>
-      <c r="N18" s="379"/>
-      <c r="O18" s="379"/>
-      <c r="P18" s="379"/>
-      <c r="Q18" s="379"/>
+      <c r="D18" s="330"/>
+      <c r="E18" s="330"/>
+      <c r="F18" s="330"/>
+      <c r="G18" s="330"/>
+      <c r="H18" s="330"/>
+      <c r="I18" s="330"/>
+      <c r="J18" s="330"/>
+      <c r="K18" s="330"/>
+      <c r="L18" s="330"/>
+      <c r="M18" s="330"/>
+      <c r="N18" s="330"/>
+      <c r="O18" s="330"/>
+      <c r="P18" s="330"/>
+      <c r="Q18" s="330"/>
     </row>
     <row r="19" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A19" s="379"/>
-      <c r="B19" s="379"/>
-      <c r="C19" s="379" t="s">
+      <c r="A19" s="330"/>
+      <c r="B19" s="330"/>
+      <c r="C19" s="330" t="s">
         <v>394</v>
       </c>
-      <c r="D19" s="379"/>
-      <c r="E19" s="379"/>
-      <c r="F19" s="379"/>
-      <c r="G19" s="379"/>
-      <c r="H19" s="379"/>
-      <c r="I19" s="379"/>
-      <c r="J19" s="379"/>
-      <c r="K19" s="379"/>
-      <c r="L19" s="379"/>
-      <c r="M19" s="379"/>
-      <c r="N19" s="379"/>
-      <c r="O19" s="379"/>
-      <c r="P19" s="379"/>
-      <c r="Q19" s="379"/>
+      <c r="D19" s="330"/>
+      <c r="E19" s="330"/>
+      <c r="F19" s="330"/>
+      <c r="G19" s="330"/>
+      <c r="H19" s="330"/>
+      <c r="I19" s="330"/>
+      <c r="J19" s="330"/>
+      <c r="K19" s="330"/>
+      <c r="L19" s="330"/>
+      <c r="M19" s="330"/>
+      <c r="N19" s="330"/>
+      <c r="O19" s="330"/>
+      <c r="P19" s="330"/>
+      <c r="Q19" s="330"/>
     </row>
     <row r="20" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A20" s="379"/>
-      <c r="B20" s="379" t="s">
+      <c r="A20" s="330"/>
+      <c r="B20" s="330" t="s">
         <v>395</v>
       </c>
-      <c r="C20" s="379" t="s">
+      <c r="C20" s="330" t="s">
         <v>396</v>
       </c>
-      <c r="D20" s="379"/>
-      <c r="E20" s="379"/>
-      <c r="F20" s="379"/>
-      <c r="G20" s="379">
+      <c r="D20" s="330"/>
+      <c r="E20" s="330"/>
+      <c r="F20" s="330"/>
+      <c r="G20" s="330">
         <v>51.5</v>
       </c>
-      <c r="H20" s="379"/>
-      <c r="I20" s="379"/>
-      <c r="J20" s="379"/>
-      <c r="K20" s="379">
+      <c r="H20" s="330"/>
+      <c r="I20" s="330"/>
+      <c r="J20" s="330"/>
+      <c r="K20" s="330">
         <v>51.5</v>
       </c>
-      <c r="L20" s="379">
+      <c r="L20" s="330">
         <v>100</v>
       </c>
-      <c r="M20" s="379"/>
-      <c r="N20" s="379"/>
-      <c r="O20" s="379"/>
-      <c r="P20" s="379"/>
-      <c r="Q20" s="379"/>
+      <c r="M20" s="330"/>
+      <c r="N20" s="330"/>
+      <c r="O20" s="330"/>
+      <c r="P20" s="330"/>
+      <c r="Q20" s="330"/>
     </row>
     <row r="21" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A21" s="379"/>
-      <c r="B21" s="379"/>
-      <c r="C21" s="379" t="s">
+      <c r="A21" s="330"/>
+      <c r="B21" s="330"/>
+      <c r="C21" s="330" t="s">
         <v>394</v>
       </c>
-      <c r="D21" s="379"/>
-      <c r="E21" s="379"/>
-      <c r="F21" s="379"/>
-      <c r="G21" s="379">
+      <c r="D21" s="330"/>
+      <c r="E21" s="330"/>
+      <c r="F21" s="330"/>
+      <c r="G21" s="330">
         <v>30</v>
       </c>
-      <c r="H21" s="379"/>
-      <c r="I21" s="379"/>
-      <c r="J21" s="379"/>
-      <c r="K21" s="379">
+      <c r="H21" s="330"/>
+      <c r="I21" s="330"/>
+      <c r="J21" s="330"/>
+      <c r="K21" s="330">
         <f>K20+30</f>
         <v>81.5</v>
       </c>
-      <c r="L21" s="400">
+      <c r="L21" s="351">
         <f>(K21*L20)/K20</f>
         <v>158.25242718446603</v>
       </c>
-      <c r="M21" s="379" t="s">
+      <c r="M21" s="330" t="s">
         <v>438</v>
       </c>
-      <c r="N21" s="379"/>
-      <c r="O21" s="379"/>
-      <c r="P21" s="379"/>
-      <c r="Q21" s="379"/>
+      <c r="N21" s="330"/>
+      <c r="O21" s="330"/>
+      <c r="P21" s="330"/>
+      <c r="Q21" s="330"/>
     </row>
     <row r="22" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A22" s="379"/>
-      <c r="B22" s="379"/>
-      <c r="C22" s="379"/>
-      <c r="D22" s="379"/>
-      <c r="E22" s="379"/>
-      <c r="F22" s="379"/>
-      <c r="G22" s="379">
+      <c r="A22" s="330"/>
+      <c r="B22" s="330"/>
+      <c r="C22" s="330"/>
+      <c r="D22" s="330"/>
+      <c r="E22" s="330"/>
+      <c r="F22" s="330"/>
+      <c r="G22" s="330">
         <v>35</v>
       </c>
-      <c r="H22" s="379"/>
-      <c r="I22" s="379"/>
-      <c r="J22" s="379"/>
-      <c r="K22" s="379">
+      <c r="H22" s="330"/>
+      <c r="I22" s="330"/>
+      <c r="J22" s="330"/>
+      <c r="K22" s="330">
         <v>35</v>
       </c>
-      <c r="L22" s="379"/>
-      <c r="M22" s="379"/>
-      <c r="N22" s="379"/>
-      <c r="O22" s="379"/>
-      <c r="P22" s="379"/>
-      <c r="Q22" s="379"/>
+      <c r="L22" s="330"/>
+      <c r="M22" s="330"/>
+      <c r="N22" s="330"/>
+      <c r="O22" s="330"/>
+      <c r="P22" s="330"/>
+      <c r="Q22" s="330"/>
     </row>
     <row r="23" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A23" s="379"/>
-      <c r="B23" s="379"/>
-      <c r="C23" s="379"/>
-      <c r="D23" s="379"/>
-      <c r="E23" s="379"/>
-      <c r="F23" s="379"/>
-      <c r="G23" s="379">
+      <c r="A23" s="330"/>
+      <c r="B23" s="330"/>
+      <c r="C23" s="330"/>
+      <c r="D23" s="330"/>
+      <c r="E23" s="330"/>
+      <c r="F23" s="330"/>
+      <c r="G23" s="330">
         <v>0.6</v>
       </c>
-      <c r="H23" s="379">
+      <c r="H23" s="330">
         <f>(G20+G21)*G23</f>
         <v>48.9</v>
       </c>
-      <c r="I23" s="379">
+      <c r="I23" s="330">
         <f>H23-G20</f>
         <v>-2.6000000000000014</v>
       </c>
-      <c r="J23" s="379"/>
-      <c r="K23" s="379">
+      <c r="J23" s="330"/>
+      <c r="K23" s="330">
         <v>0.6</v>
       </c>
-      <c r="L23" s="379">
+      <c r="L23" s="330">
         <f>(K20+K21)</f>
         <v>133</v>
       </c>
-      <c r="M23" s="379">
+      <c r="M23" s="330">
         <f>L23-K20</f>
         <v>81.5</v>
       </c>
-      <c r="N23" s="379"/>
-      <c r="O23" s="379"/>
-      <c r="P23" s="379"/>
-      <c r="Q23" s="379"/>
+      <c r="N23" s="330"/>
+      <c r="O23" s="330"/>
+      <c r="P23" s="330"/>
+      <c r="Q23" s="330"/>
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.2">
       <c r="H24">
@@ -40081,6 +40083,890 @@
       <c r="L24">
         <f>K20-L23</f>
         <v>-81.5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="B29" s="172" t="s">
+        <v>276</v>
+      </c>
+      <c r="C29" s="173"/>
+      <c r="D29" s="173"/>
+      <c r="E29" s="173"/>
+      <c r="F29" s="173"/>
+      <c r="G29" s="173"/>
+      <c r="H29" s="173"/>
+      <c r="I29" s="173"/>
+      <c r="J29" s="173"/>
+      <c r="K29" s="173"/>
+      <c r="L29" s="173"/>
+      <c r="M29" s="173"/>
+      <c r="N29" s="173"/>
+      <c r="O29" s="173"/>
+    </row>
+    <row r="30" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="C30" s="2"/>
+      <c r="D30" s="2"/>
+      <c r="E30" s="2"/>
+      <c r="F30" s="2"/>
+      <c r="G30" s="2"/>
+    </row>
+    <row r="31" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="B31" t="s">
+        <v>216</v>
+      </c>
+      <c r="C31" s="2"/>
+      <c r="D31" s="2"/>
+      <c r="E31" s="2"/>
+      <c r="F31" s="2"/>
+      <c r="G31" s="2"/>
+    </row>
+    <row r="32" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="B32" s="125" t="s">
+        <v>8</v>
+      </c>
+      <c r="C32" s="117" t="s">
+        <v>14</v>
+      </c>
+      <c r="D32" s="117" t="s">
+        <v>15</v>
+      </c>
+      <c r="E32" s="117" t="s">
+        <v>29</v>
+      </c>
+      <c r="F32" s="117" t="s">
+        <v>16</v>
+      </c>
+      <c r="G32" s="117" t="s">
+        <v>59</v>
+      </c>
+      <c r="H32" s="117" t="s">
+        <v>17</v>
+      </c>
+      <c r="I32" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="J32" s="122" t="s">
+        <v>214</v>
+      </c>
+      <c r="K32" s="120" t="s">
+        <v>210</v>
+      </c>
+      <c r="L32" s="117" t="s">
+        <v>211</v>
+      </c>
+      <c r="M32" s="118" t="s">
+        <v>209</v>
+      </c>
+      <c r="N32" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="33" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B33" t="s">
+        <v>213</v>
+      </c>
+      <c r="C33" s="15">
+        <v>4</v>
+      </c>
+      <c r="D33" s="15">
+        <v>1</v>
+      </c>
+      <c r="E33" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="F33" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="G33" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="H33" s="15">
+        <f t="shared" ref="H33" si="0">J33*I33</f>
+        <v>42.274999999999999</v>
+      </c>
+      <c r="I33" s="119">
+        <v>0.95</v>
+      </c>
+      <c r="J33" s="122">
+        <f>M33-(K33+L33)</f>
+        <v>44.5</v>
+      </c>
+      <c r="K33" s="121">
+        <v>7</v>
+      </c>
+      <c r="L33" s="42">
+        <v>0</v>
+      </c>
+      <c r="M33" s="42">
+        <v>51.5</v>
+      </c>
+    </row>
+    <row r="34" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="C34" s="2"/>
+      <c r="D34" s="2"/>
+      <c r="E34" s="2"/>
+      <c r="F34" s="2"/>
+      <c r="G34" s="2"/>
+    </row>
+    <row r="35" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="C35" s="2"/>
+      <c r="D35" s="2"/>
+      <c r="E35" s="2"/>
+      <c r="F35" s="2"/>
+      <c r="G35" s="2"/>
+      <c r="H35">
+        <v>36.700000000000003</v>
+      </c>
+      <c r="J35">
+        <v>39.700000000000003</v>
+      </c>
+      <c r="K35">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="36" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="C36" s="2"/>
+      <c r="D36" s="2"/>
+      <c r="E36" s="2"/>
+      <c r="F36" s="2"/>
+      <c r="G36" s="2"/>
+      <c r="J36" s="124">
+        <f>(J35*K36)/K35</f>
+        <v>44.111111111111114</v>
+      </c>
+      <c r="K36">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="37" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B37" s="125" t="s">
+        <v>163</v>
+      </c>
+      <c r="C37" s="117" t="s">
+        <v>14</v>
+      </c>
+      <c r="D37" s="117" t="s">
+        <v>15</v>
+      </c>
+      <c r="E37" s="117" t="s">
+        <v>29</v>
+      </c>
+      <c r="F37" s="117" t="s">
+        <v>16</v>
+      </c>
+      <c r="G37" s="117" t="s">
+        <v>59</v>
+      </c>
+      <c r="H37" s="117" t="s">
+        <v>17</v>
+      </c>
+      <c r="I37" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="J37" s="122" t="s">
+        <v>214</v>
+      </c>
+      <c r="K37" s="120" t="s">
+        <v>210</v>
+      </c>
+      <c r="L37" s="117" t="s">
+        <v>211</v>
+      </c>
+      <c r="M37" s="118" t="s">
+        <v>209</v>
+      </c>
+      <c r="N37" s="123" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="38" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B38" t="s">
+        <v>314</v>
+      </c>
+      <c r="C38" s="15">
+        <v>4</v>
+      </c>
+      <c r="D38" s="15">
+        <v>1</v>
+      </c>
+      <c r="E38" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="F38" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="G38" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="H38" s="15">
+        <f t="shared" ref="H38" si="1">J38*I38</f>
+        <v>24.3</v>
+      </c>
+      <c r="I38" s="119">
+        <v>0.9</v>
+      </c>
+      <c r="J38" s="122">
+        <f>(K38+L38)</f>
+        <v>27</v>
+      </c>
+      <c r="K38" s="121">
+        <v>0</v>
+      </c>
+      <c r="L38" s="42">
+        <v>27</v>
+      </c>
+      <c r="M38" s="42">
+        <f>M33</f>
+        <v>51.5</v>
+      </c>
+      <c r="N38" s="126" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="39" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
+      <c r="E39" s="2"/>
+      <c r="F39" s="2"/>
+      <c r="G39" s="2"/>
+    </row>
+    <row r="40" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B40" s="125" t="s">
+        <v>315</v>
+      </c>
+      <c r="C40" s="117" t="s">
+        <v>14</v>
+      </c>
+      <c r="D40" s="117" t="s">
+        <v>15</v>
+      </c>
+      <c r="E40" s="117" t="s">
+        <v>29</v>
+      </c>
+      <c r="F40" s="117" t="s">
+        <v>16</v>
+      </c>
+      <c r="G40" s="117" t="s">
+        <v>59</v>
+      </c>
+      <c r="H40" s="117" t="s">
+        <v>17</v>
+      </c>
+      <c r="I40" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="J40" s="122" t="s">
+        <v>214</v>
+      </c>
+      <c r="K40" s="120" t="s">
+        <v>210</v>
+      </c>
+      <c r="L40" s="117" t="s">
+        <v>211</v>
+      </c>
+      <c r="M40" s="118" t="s">
+        <v>209</v>
+      </c>
+      <c r="N40" s="123" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="41" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B41" t="s">
+        <v>311</v>
+      </c>
+      <c r="C41" s="15">
+        <v>4</v>
+      </c>
+      <c r="D41" s="15">
+        <v>7</v>
+      </c>
+      <c r="E41" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="F41" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="G41" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="H41" s="15">
+        <f t="shared" ref="H41" si="2">J41*I41</f>
+        <v>-16.099999999999998</v>
+      </c>
+      <c r="I41" s="119">
+        <v>0.7</v>
+      </c>
+      <c r="J41" s="122">
+        <f>(K41+L41)</f>
+        <v>-23</v>
+      </c>
+      <c r="K41" s="121">
+        <v>-23</v>
+      </c>
+      <c r="L41" s="42">
+        <v>0</v>
+      </c>
+      <c r="M41" s="42">
+        <f>M33</f>
+        <v>51.5</v>
+      </c>
+      <c r="N41" s="126" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="42" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="C42" s="2"/>
+      <c r="D42" s="2"/>
+      <c r="E42" s="2"/>
+      <c r="F42" s="2"/>
+      <c r="G42" s="2"/>
+    </row>
+    <row r="43" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B43" s="125" t="s">
+        <v>163</v>
+      </c>
+      <c r="C43" s="117" t="s">
+        <v>14</v>
+      </c>
+      <c r="D43" s="117" t="s">
+        <v>15</v>
+      </c>
+      <c r="E43" s="117" t="s">
+        <v>29</v>
+      </c>
+      <c r="F43" s="117" t="s">
+        <v>16</v>
+      </c>
+      <c r="G43" s="117" t="s">
+        <v>59</v>
+      </c>
+      <c r="H43" s="117" t="s">
+        <v>17</v>
+      </c>
+      <c r="I43" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="J43" s="122" t="s">
+        <v>214</v>
+      </c>
+      <c r="K43" s="120" t="s">
+        <v>210</v>
+      </c>
+      <c r="L43" s="117" t="s">
+        <v>211</v>
+      </c>
+      <c r="M43" s="118" t="s">
+        <v>209</v>
+      </c>
+      <c r="N43" s="123" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="44" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B44" t="s">
+        <v>316</v>
+      </c>
+      <c r="C44" s="15">
+        <v>4</v>
+      </c>
+      <c r="D44" s="15">
+        <v>1</v>
+      </c>
+      <c r="E44" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="F44" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="G44" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="H44" s="15">
+        <f t="shared" ref="H44" si="3">J44*I44</f>
+        <v>39.9</v>
+      </c>
+      <c r="I44" s="119">
+        <v>0.95</v>
+      </c>
+      <c r="J44" s="122">
+        <f>(K44+L44)</f>
+        <v>42</v>
+      </c>
+      <c r="K44" s="121">
+        <v>0</v>
+      </c>
+      <c r="L44" s="42">
+        <v>42</v>
+      </c>
+      <c r="M44" s="42">
+        <f>M33</f>
+        <v>51.5</v>
+      </c>
+      <c r="N44" s="126" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="45" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="C45" s="2"/>
+      <c r="D45" s="2"/>
+      <c r="E45" s="2"/>
+      <c r="F45" s="2"/>
+      <c r="G45" s="2"/>
+    </row>
+    <row r="46" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="C46" s="2"/>
+      <c r="D46" s="2"/>
+      <c r="E46" s="2"/>
+      <c r="F46" s="2"/>
+      <c r="G46" s="2"/>
+    </row>
+    <row r="47" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B47" s="125" t="s">
+        <v>8</v>
+      </c>
+      <c r="C47" s="117" t="s">
+        <v>14</v>
+      </c>
+      <c r="D47" s="117" t="s">
+        <v>15</v>
+      </c>
+      <c r="E47" s="117" t="s">
+        <v>29</v>
+      </c>
+      <c r="F47" s="117" t="s">
+        <v>16</v>
+      </c>
+      <c r="G47" s="117" t="s">
+        <v>59</v>
+      </c>
+      <c r="H47" s="117" t="s">
+        <v>17</v>
+      </c>
+      <c r="I47" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="J47" s="122" t="s">
+        <v>214</v>
+      </c>
+      <c r="K47" s="120" t="s">
+        <v>210</v>
+      </c>
+      <c r="L47" s="117" t="s">
+        <v>211</v>
+      </c>
+      <c r="M47" s="118" t="s">
+        <v>209</v>
+      </c>
+      <c r="N47" s="123" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="48" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B48" t="s">
+        <v>277</v>
+      </c>
+      <c r="C48" s="15">
+        <v>4</v>
+      </c>
+      <c r="D48" s="15">
+        <v>1</v>
+      </c>
+      <c r="E48" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="F48" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="G48" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="H48" s="15">
+        <v>6</v>
+      </c>
+      <c r="I48" s="119">
+        <v>0.9</v>
+      </c>
+      <c r="J48" s="122">
+        <f>(K48+L48)</f>
+        <v>7</v>
+      </c>
+      <c r="K48" s="121">
+        <v>0</v>
+      </c>
+      <c r="L48" s="42">
+        <v>7</v>
+      </c>
+      <c r="M48" s="42">
+        <f>M33</f>
+        <v>51.5</v>
+      </c>
+      <c r="N48" s="126" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="49" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="C49" s="2"/>
+      <c r="D49" s="2"/>
+      <c r="E49" s="2"/>
+      <c r="F49" s="2"/>
+      <c r="G49" s="2"/>
+    </row>
+    <row r="50" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B50" s="125" t="s">
+        <v>8</v>
+      </c>
+      <c r="C50" s="117" t="s">
+        <v>14</v>
+      </c>
+      <c r="D50" s="117" t="s">
+        <v>15</v>
+      </c>
+      <c r="E50" s="117" t="s">
+        <v>29</v>
+      </c>
+      <c r="F50" s="117" t="s">
+        <v>16</v>
+      </c>
+      <c r="G50" s="117" t="s">
+        <v>59</v>
+      </c>
+      <c r="H50" s="117" t="s">
+        <v>17</v>
+      </c>
+      <c r="I50" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="J50" s="122" t="s">
+        <v>214</v>
+      </c>
+      <c r="K50" s="120" t="s">
+        <v>210</v>
+      </c>
+      <c r="L50" s="117" t="s">
+        <v>211</v>
+      </c>
+      <c r="M50" s="118" t="s">
+        <v>209</v>
+      </c>
+      <c r="N50" s="123" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="51" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B51" t="s">
+        <v>278</v>
+      </c>
+      <c r="C51" s="15">
+        <v>4</v>
+      </c>
+      <c r="D51" s="15">
+        <v>1</v>
+      </c>
+      <c r="E51" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="F51" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="G51" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="H51" s="15">
+        <v>10</v>
+      </c>
+      <c r="I51" s="119">
+        <v>0.8</v>
+      </c>
+      <c r="J51" s="122">
+        <f>(K51+L51)</f>
+        <v>13.5</v>
+      </c>
+      <c r="K51" s="121">
+        <v>0</v>
+      </c>
+      <c r="L51" s="42">
+        <v>13.5</v>
+      </c>
+      <c r="M51" s="42">
+        <f>M33</f>
+        <v>51.5</v>
+      </c>
+      <c r="N51" s="126" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="52" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="C52" s="2"/>
+      <c r="D52" s="2"/>
+      <c r="E52" s="2"/>
+      <c r="F52" s="2"/>
+      <c r="G52" s="2"/>
+    </row>
+    <row r="53" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B53" s="125" t="s">
+        <v>8</v>
+      </c>
+      <c r="C53" s="117" t="s">
+        <v>14</v>
+      </c>
+      <c r="D53" s="117" t="s">
+        <v>15</v>
+      </c>
+      <c r="E53" s="117" t="s">
+        <v>29</v>
+      </c>
+      <c r="F53" s="117" t="s">
+        <v>16</v>
+      </c>
+      <c r="G53" s="117" t="s">
+        <v>59</v>
+      </c>
+      <c r="H53" s="117" t="s">
+        <v>17</v>
+      </c>
+      <c r="I53" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="J53" s="122" t="s">
+        <v>214</v>
+      </c>
+      <c r="K53" s="120" t="s">
+        <v>210</v>
+      </c>
+      <c r="L53" s="117" t="s">
+        <v>211</v>
+      </c>
+      <c r="M53" s="118" t="s">
+        <v>209</v>
+      </c>
+      <c r="N53" s="123" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="54" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B54" t="s">
+        <v>279</v>
+      </c>
+      <c r="C54" s="15">
+        <v>4</v>
+      </c>
+      <c r="D54" s="15">
+        <v>1</v>
+      </c>
+      <c r="E54" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="F54" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="G54" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="H54" s="15">
+        <v>10</v>
+      </c>
+      <c r="I54" s="119">
+        <v>0.9</v>
+      </c>
+      <c r="J54" s="122">
+        <f>(K54+L54)</f>
+        <v>13.5</v>
+      </c>
+      <c r="K54" s="121">
+        <v>0</v>
+      </c>
+      <c r="L54" s="42">
+        <v>13.5</v>
+      </c>
+      <c r="M54" s="42">
+        <f>M5</f>
+        <v>0</v>
+      </c>
+      <c r="N54" s="126" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="55" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="C55" s="2"/>
+      <c r="D55" s="2"/>
+      <c r="E55" s="2"/>
+      <c r="F55" s="2"/>
+      <c r="G55" s="2"/>
+    </row>
+    <row r="56" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B56" s="125" t="s">
+        <v>8</v>
+      </c>
+      <c r="C56" s="117" t="s">
+        <v>14</v>
+      </c>
+      <c r="D56" s="117" t="s">
+        <v>15</v>
+      </c>
+      <c r="E56" s="117" t="s">
+        <v>29</v>
+      </c>
+      <c r="F56" s="117" t="s">
+        <v>16</v>
+      </c>
+      <c r="G56" s="117" t="s">
+        <v>59</v>
+      </c>
+      <c r="H56" s="117" t="s">
+        <v>17</v>
+      </c>
+      <c r="I56" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="J56" s="122" t="s">
+        <v>214</v>
+      </c>
+      <c r="K56" s="120" t="s">
+        <v>210</v>
+      </c>
+      <c r="L56" s="117" t="s">
+        <v>211</v>
+      </c>
+      <c r="M56" s="118" t="s">
+        <v>209</v>
+      </c>
+      <c r="N56" s="123" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="57" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B57" t="s">
+        <v>280</v>
+      </c>
+      <c r="C57" s="15">
+        <v>4</v>
+      </c>
+      <c r="D57" s="15">
+        <v>1</v>
+      </c>
+      <c r="E57" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="F57" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="G57" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="H57" s="15">
+        <v>10</v>
+      </c>
+      <c r="I57" s="119">
+        <v>0.9</v>
+      </c>
+      <c r="J57" s="122">
+        <f>(K57+L57)</f>
+        <v>13.5</v>
+      </c>
+      <c r="K57" s="121">
+        <v>0</v>
+      </c>
+      <c r="L57" s="42">
+        <v>13.5</v>
+      </c>
+      <c r="M57" s="42">
+        <f>M33</f>
+        <v>51.5</v>
+      </c>
+      <c r="N57" s="126" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="58" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="C58" s="2"/>
+      <c r="D58" s="2"/>
+      <c r="E58" s="2"/>
+      <c r="F58" s="2"/>
+      <c r="G58" s="2"/>
+    </row>
+    <row r="59" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B59" s="125" t="s">
+        <v>8</v>
+      </c>
+      <c r="C59" s="117" t="s">
+        <v>14</v>
+      </c>
+      <c r="D59" s="117" t="s">
+        <v>15</v>
+      </c>
+      <c r="E59" s="117" t="s">
+        <v>29</v>
+      </c>
+      <c r="F59" s="117" t="s">
+        <v>16</v>
+      </c>
+      <c r="G59" s="117" t="s">
+        <v>59</v>
+      </c>
+      <c r="H59" s="117" t="s">
+        <v>17</v>
+      </c>
+      <c r="I59" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="J59" s="122" t="s">
+        <v>214</v>
+      </c>
+      <c r="K59" s="120" t="s">
+        <v>210</v>
+      </c>
+      <c r="L59" s="117" t="s">
+        <v>211</v>
+      </c>
+      <c r="M59" s="118" t="s">
+        <v>209</v>
+      </c>
+      <c r="N59" s="123" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="60" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B60" t="s">
+        <v>485</v>
+      </c>
+      <c r="C60" s="15">
+        <v>4</v>
+      </c>
+      <c r="D60" s="15">
+        <v>1</v>
+      </c>
+      <c r="E60" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="F60" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="G60" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="H60" s="15">
+        <v>10</v>
+      </c>
+      <c r="I60" s="119">
+        <v>0.9</v>
+      </c>
+      <c r="J60" s="122">
+        <f>(K60+L60)</f>
+        <v>13.5</v>
+      </c>
+      <c r="K60" s="121">
+        <v>0</v>
+      </c>
+      <c r="L60" s="42">
+        <v>13.5</v>
+      </c>
+      <c r="M60" s="42">
+        <f>M33</f>
+        <v>51.5</v>
+      </c>
+      <c r="N60" s="126" t="s">
+        <v>218</v>
       </c>
     </row>
   </sheetData>
@@ -40244,18 +41130,18 @@
       <c r="K12" s="183" t="s">
         <v>160</v>
       </c>
-      <c r="Q12" s="337" t="s">
+      <c r="Q12" s="359" t="s">
         <v>344</v>
       </c>
-      <c r="R12" s="338"/>
+      <c r="R12" s="360"/>
       <c r="Y12" s="186"/>
       <c r="Z12" t="s">
         <v>417</v>
       </c>
-      <c r="AC12" s="337" t="s">
+      <c r="AC12" s="359" t="s">
         <v>344</v>
       </c>
-      <c r="AD12" s="338"/>
+      <c r="AD12" s="360"/>
       <c r="AE12" t="s">
         <v>243</v>
       </c>
@@ -40972,17 +41858,17 @@
       </c>
     </row>
     <row r="38" spans="1:29" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="336" t="s">
+      <c r="A38" s="358" t="s">
         <v>397</v>
       </c>
-      <c r="B38" s="336"/>
-      <c r="C38" s="336"/>
-      <c r="F38" s="336" t="s">
+      <c r="B38" s="358"/>
+      <c r="C38" s="358"/>
+      <c r="F38" s="358" t="s">
         <v>403</v>
       </c>
-      <c r="G38" s="336"/>
-      <c r="H38" s="336"/>
-      <c r="I38" s="336"/>
+      <c r="G38" s="358"/>
+      <c r="H38" s="358"/>
+      <c r="I38" s="358"/>
       <c r="M38" t="s">
         <v>355</v>
       </c>
@@ -41012,31 +41898,31 @@
       <c r="M39" s="210" t="s">
         <v>357</v>
       </c>
-      <c r="N39" s="339" t="s">
+      <c r="N39" s="361" t="s">
         <v>356</v>
       </c>
-      <c r="O39" s="340"/>
-      <c r="P39" s="341" t="s">
+      <c r="O39" s="362"/>
+      <c r="P39" s="363" t="s">
         <v>456</v>
       </c>
-      <c r="Q39" s="342"/>
-      <c r="R39" s="343"/>
-      <c r="U39" s="344" t="s">
+      <c r="Q39" s="364"/>
+      <c r="R39" s="365"/>
+      <c r="U39" s="366" t="s">
         <v>410</v>
       </c>
-      <c r="V39" s="345"/>
+      <c r="V39" s="367"/>
       <c r="X39" s="210" t="s">
         <v>357</v>
       </c>
-      <c r="Y39" s="339" t="s">
+      <c r="Y39" s="361" t="s">
         <v>356</v>
       </c>
-      <c r="Z39" s="340"/>
-      <c r="AA39" s="341" t="s">
+      <c r="Z39" s="362"/>
+      <c r="AA39" s="363" t="s">
         <v>456</v>
       </c>
-      <c r="AB39" s="342"/>
-      <c r="AC39" s="343"/>
+      <c r="AB39" s="364"/>
+      <c r="AC39" s="365"/>
     </row>
     <row r="40" spans="1:29" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A40" s="58" t="s">
@@ -41078,8 +41964,8 @@
         <f>(P40*N40)+(Q40*O40)+0</f>
         <v>0</v>
       </c>
-      <c r="U40" s="346"/>
-      <c r="V40" s="347"/>
+      <c r="U40" s="368"/>
+      <c r="V40" s="369"/>
       <c r="X40" s="211" t="s">
         <v>146</v>
       </c>
@@ -41533,10 +42419,10 @@
         <v>3</v>
       </c>
       <c r="W51" s="214"/>
-      <c r="X51" s="334" t="s">
+      <c r="X51" s="356" t="s">
         <v>165</v>
       </c>
-      <c r="Y51" s="335"/>
+      <c r="Y51" s="357"/>
     </row>
     <row r="52" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
@@ -41986,79 +42872,79 @@
       </c>
     </row>
     <row r="35" spans="2:36" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="M35" s="341" t="s">
+      <c r="M35" s="363" t="s">
         <v>135</v>
       </c>
-      <c r="N35" s="342"/>
-      <c r="O35" s="342"/>
-      <c r="P35" s="343"/>
-      <c r="R35" s="341" t="s">
+      <c r="N35" s="364"/>
+      <c r="O35" s="364"/>
+      <c r="P35" s="365"/>
+      <c r="R35" s="363" t="s">
         <v>135</v>
       </c>
-      <c r="S35" s="342"/>
-      <c r="T35" s="342"/>
-      <c r="U35" s="343"/>
-      <c r="W35" s="341" t="s">
+      <c r="S35" s="364"/>
+      <c r="T35" s="364"/>
+      <c r="U35" s="365"/>
+      <c r="W35" s="363" t="s">
         <v>135</v>
       </c>
-      <c r="X35" s="342"/>
-      <c r="Y35" s="342"/>
-      <c r="Z35" s="343"/>
-      <c r="AB35" s="341" t="s">
+      <c r="X35" s="364"/>
+      <c r="Y35" s="364"/>
+      <c r="Z35" s="365"/>
+      <c r="AB35" s="363" t="s">
         <v>135</v>
       </c>
-      <c r="AC35" s="342"/>
-      <c r="AD35" s="342"/>
-      <c r="AE35" s="343"/>
-      <c r="AG35" s="341" t="s">
+      <c r="AC35" s="364"/>
+      <c r="AD35" s="364"/>
+      <c r="AE35" s="365"/>
+      <c r="AG35" s="363" t="s">
         <v>135</v>
       </c>
-      <c r="AH35" s="342"/>
-      <c r="AI35" s="342"/>
-      <c r="AJ35" s="343"/>
+      <c r="AH35" s="364"/>
+      <c r="AI35" s="364"/>
+      <c r="AJ35" s="365"/>
     </row>
     <row r="36" spans="2:36" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="M36" s="341">
+      <c r="M36" s="363">
         <v>42</v>
       </c>
-      <c r="N36" s="342"/>
-      <c r="O36" s="342"/>
+      <c r="N36" s="364"/>
+      <c r="O36" s="364"/>
       <c r="P36" s="326" t="s">
         <v>147</v>
       </c>
-      <c r="R36" s="341">
+      <c r="R36" s="363">
         <f>M36+1</f>
         <v>43</v>
       </c>
-      <c r="S36" s="342"/>
-      <c r="T36" s="342"/>
+      <c r="S36" s="364"/>
+      <c r="T36" s="364"/>
       <c r="U36" s="326" t="s">
         <v>147</v>
       </c>
-      <c r="W36" s="341">
+      <c r="W36" s="363">
         <f>R36+1</f>
         <v>44</v>
       </c>
-      <c r="X36" s="342"/>
-      <c r="Y36" s="342"/>
+      <c r="X36" s="364"/>
+      <c r="Y36" s="364"/>
       <c r="Z36" s="326" t="s">
         <v>147</v>
       </c>
-      <c r="AB36" s="341">
+      <c r="AB36" s="363">
         <f>W36+1</f>
         <v>45</v>
       </c>
-      <c r="AC36" s="342"/>
-      <c r="AD36" s="342"/>
+      <c r="AC36" s="364"/>
+      <c r="AD36" s="364"/>
       <c r="AE36" s="326" t="s">
         <v>147</v>
       </c>
-      <c r="AG36" s="341">
+      <c r="AG36" s="363">
         <f>AB36+1</f>
         <v>46</v>
       </c>
-      <c r="AH36" s="342"/>
-      <c r="AI36" s="342"/>
+      <c r="AH36" s="364"/>
+      <c r="AI36" s="364"/>
       <c r="AJ36" s="326" t="s">
         <v>147</v>
       </c>
@@ -43476,10 +44362,10 @@
       </c>
     </row>
     <row r="70" spans="11:14" x14ac:dyDescent="0.2">
-      <c r="K70" s="348" t="s">
+      <c r="K70" s="370" t="s">
         <v>467</v>
       </c>
-      <c r="L70" s="349"/>
+      <c r="L70" s="371"/>
       <c r="M70" s="108">
         <f>P39+U39+Z39+AE39+AJ39</f>
         <v>208</v>
@@ -43490,10 +44376,10 @@
       </c>
     </row>
     <row r="71" spans="11:14" x14ac:dyDescent="0.2">
-      <c r="K71" s="350" t="s">
+      <c r="K71" s="372" t="s">
         <v>207</v>
       </c>
-      <c r="L71" s="351"/>
+      <c r="L71" s="373"/>
       <c r="M71" s="302"/>
       <c r="N71" s="298">
         <f t="shared" ref="N71:N72" si="12">P39+U39+Z39+AE39+AJ39</f>
@@ -43501,10 +44387,10 @@
       </c>
     </row>
     <row r="72" spans="11:14" x14ac:dyDescent="0.2">
-      <c r="K72" s="350" t="s">
+      <c r="K72" s="372" t="s">
         <v>196</v>
       </c>
-      <c r="L72" s="351"/>
+      <c r="L72" s="373"/>
       <c r="M72" s="302"/>
       <c r="N72" s="298">
         <f t="shared" si="12"/>
@@ -43513,11 +44399,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="K70:L70"/>
-    <mergeCell ref="K71:L71"/>
-    <mergeCell ref="K72:L72"/>
-    <mergeCell ref="M36:O36"/>
-    <mergeCell ref="R36:T36"/>
     <mergeCell ref="W36:Y36"/>
     <mergeCell ref="AB36:AD36"/>
     <mergeCell ref="AG36:AI36"/>
@@ -43526,6 +44407,11 @@
     <mergeCell ref="W35:Z35"/>
     <mergeCell ref="AB35:AE35"/>
     <mergeCell ref="AG35:AJ35"/>
+    <mergeCell ref="K70:L70"/>
+    <mergeCell ref="K71:L71"/>
+    <mergeCell ref="K72:L72"/>
+    <mergeCell ref="M36:O36"/>
+    <mergeCell ref="R36:T36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -43736,26 +44622,26 @@
       <c r="G11" s="27" t="s">
         <v>95</v>
       </c>
-      <c r="M11" s="357" t="s">
+      <c r="M11" s="390" t="s">
         <v>135</v>
       </c>
-      <c r="N11" s="358"/>
-      <c r="O11" s="359"/>
-      <c r="Q11" s="357" t="s">
+      <c r="N11" s="391"/>
+      <c r="O11" s="392"/>
+      <c r="Q11" s="390" t="s">
         <v>135</v>
       </c>
-      <c r="R11" s="358"/>
-      <c r="S11" s="359"/>
-      <c r="U11" s="357" t="s">
+      <c r="R11" s="391"/>
+      <c r="S11" s="392"/>
+      <c r="U11" s="390" t="s">
         <v>135</v>
       </c>
-      <c r="V11" s="358"/>
-      <c r="W11" s="359"/>
-      <c r="Y11" s="357" t="s">
+      <c r="V11" s="391"/>
+      <c r="W11" s="392"/>
+      <c r="Y11" s="390" t="s">
         <v>135</v>
       </c>
-      <c r="Z11" s="358"/>
-      <c r="AA11" s="359"/>
+      <c r="Z11" s="391"/>
+      <c r="AA11" s="392"/>
     </row>
     <row r="12" spans="1:27" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B12" s="28" t="s">
@@ -43776,31 +44662,31 @@
       <c r="G12" s="28" t="s">
         <v>101</v>
       </c>
-      <c r="M12" s="355">
+      <c r="M12" s="393">
         <v>46</v>
       </c>
-      <c r="N12" s="356"/>
+      <c r="N12" s="394"/>
       <c r="O12" s="44" t="s">
         <v>147</v>
       </c>
-      <c r="Q12" s="355">
+      <c r="Q12" s="393">
         <v>47</v>
       </c>
-      <c r="R12" s="356"/>
+      <c r="R12" s="394"/>
       <c r="S12" s="44" t="s">
         <v>147</v>
       </c>
-      <c r="U12" s="355">
+      <c r="U12" s="393">
         <v>48</v>
       </c>
-      <c r="V12" s="356"/>
+      <c r="V12" s="394"/>
       <c r="W12" s="44" t="s">
         <v>147</v>
       </c>
-      <c r="Y12" s="355">
+      <c r="Y12" s="393">
         <v>49</v>
       </c>
-      <c r="Z12" s="356"/>
+      <c r="Z12" s="394"/>
       <c r="AA12" s="44" t="s">
         <v>147</v>
       </c>
@@ -45034,31 +45920,31 @@
       <c r="G66" s="27" t="s">
         <v>95</v>
       </c>
-      <c r="M66" s="357" t="s">
+      <c r="M66" s="390" t="s">
         <v>135</v>
       </c>
-      <c r="N66" s="358"/>
-      <c r="O66" s="359"/>
-      <c r="Q66" s="357" t="s">
+      <c r="N66" s="391"/>
+      <c r="O66" s="392"/>
+      <c r="Q66" s="390" t="s">
         <v>135</v>
       </c>
-      <c r="R66" s="358"/>
-      <c r="S66" s="359"/>
-      <c r="U66" s="357" t="s">
+      <c r="R66" s="391"/>
+      <c r="S66" s="392"/>
+      <c r="U66" s="390" t="s">
         <v>135</v>
       </c>
-      <c r="V66" s="358"/>
-      <c r="W66" s="359"/>
-      <c r="Y66" s="357" t="s">
+      <c r="V66" s="391"/>
+      <c r="W66" s="392"/>
+      <c r="Y66" s="390" t="s">
         <v>135</v>
       </c>
-      <c r="Z66" s="358"/>
-      <c r="AA66" s="359"/>
-      <c r="AC66" s="357" t="s">
+      <c r="Z66" s="391"/>
+      <c r="AA66" s="392"/>
+      <c r="AC66" s="390" t="s">
         <v>135</v>
       </c>
-      <c r="AD66" s="358"/>
-      <c r="AE66" s="359"/>
+      <c r="AD66" s="391"/>
+      <c r="AE66" s="392"/>
     </row>
     <row r="67" spans="1:31" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B67" s="28" t="s">
@@ -45079,38 +45965,38 @@
       <c r="G67" s="28" t="s">
         <v>101</v>
       </c>
-      <c r="M67" s="355">
+      <c r="M67" s="393">
         <v>1</v>
       </c>
-      <c r="N67" s="356"/>
+      <c r="N67" s="394"/>
       <c r="O67" s="44" t="s">
         <v>147</v>
       </c>
-      <c r="Q67" s="355">
+      <c r="Q67" s="393">
         <v>2</v>
       </c>
-      <c r="R67" s="356"/>
+      <c r="R67" s="394"/>
       <c r="S67" s="44" t="s">
         <v>147</v>
       </c>
-      <c r="U67" s="355">
+      <c r="U67" s="393">
         <v>3</v>
       </c>
-      <c r="V67" s="356"/>
+      <c r="V67" s="394"/>
       <c r="W67" s="44" t="s">
         <v>147</v>
       </c>
-      <c r="Y67" s="355">
+      <c r="Y67" s="393">
         <v>4</v>
       </c>
-      <c r="Z67" s="356"/>
+      <c r="Z67" s="394"/>
       <c r="AA67" s="44" t="s">
         <v>147</v>
       </c>
-      <c r="AC67" s="355">
+      <c r="AC67" s="393">
         <v>5</v>
       </c>
-      <c r="AD67" s="356"/>
+      <c r="AD67" s="394"/>
       <c r="AE67" s="44" t="s">
         <v>147</v>
       </c>
@@ -46229,39 +47115,39 @@
       <c r="L85" s="98" t="s">
         <v>191</v>
       </c>
-      <c r="M85" s="341"/>
-      <c r="N85" s="342"/>
-      <c r="O85" s="343"/>
+      <c r="M85" s="363"/>
+      <c r="N85" s="364"/>
+      <c r="O85" s="365"/>
       <c r="P85" s="98" t="s">
         <v>191</v>
       </c>
-      <c r="Q85" s="341"/>
-      <c r="R85" s="342"/>
-      <c r="S85" s="343"/>
+      <c r="Q85" s="363"/>
+      <c r="R85" s="364"/>
+      <c r="S85" s="365"/>
       <c r="T85" s="98" t="s">
         <v>191</v>
       </c>
-      <c r="U85" s="341" t="s">
+      <c r="U85" s="363" t="s">
         <v>192</v>
       </c>
-      <c r="V85" s="342"/>
-      <c r="W85" s="343"/>
+      <c r="V85" s="364"/>
+      <c r="W85" s="365"/>
       <c r="X85" s="98" t="s">
         <v>191</v>
       </c>
-      <c r="Y85" s="341" t="s">
+      <c r="Y85" s="363" t="s">
         <v>193</v>
       </c>
-      <c r="Z85" s="342"/>
-      <c r="AA85" s="343"/>
+      <c r="Z85" s="364"/>
+      <c r="AA85" s="365"/>
       <c r="AB85" s="98" t="s">
         <v>191</v>
       </c>
-      <c r="AC85" s="341" t="s">
+      <c r="AC85" s="363" t="s">
         <v>194</v>
       </c>
-      <c r="AD85" s="342"/>
-      <c r="AE85" s="343"/>
+      <c r="AD85" s="364"/>
+      <c r="AE85" s="365"/>
     </row>
     <row r="86" spans="2:31" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B86" s="45" t="s">
@@ -46479,21 +47365,21 @@
       </c>
     </row>
     <row r="105" spans="11:13" x14ac:dyDescent="0.2">
-      <c r="K105" s="367" t="s">
+      <c r="K105" s="388" t="s">
         <v>196</v>
       </c>
-      <c r="L105" s="368"/>
+      <c r="L105" s="389"/>
       <c r="M105" s="109">
         <f>140+260</f>
         <v>400</v>
       </c>
     </row>
     <row r="106" spans="11:13" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="K106" s="369" t="str">
+      <c r="K106" s="374" t="str">
         <f>L48</f>
         <v>Total meters November:</v>
       </c>
-      <c r="L106" s="370"/>
+      <c r="L106" s="375"/>
       <c r="M106" s="110">
         <f>M48</f>
         <v>1165</v>
@@ -46699,27 +47585,27 @@
       <c r="G136" s="27" t="s">
         <v>95</v>
       </c>
-      <c r="M136" s="357" t="s">
+      <c r="M136" s="390" t="s">
         <v>135</v>
       </c>
-      <c r="N136" s="358"/>
-      <c r="O136" s="359"/>
-      <c r="Q136" s="357" t="s">
+      <c r="N136" s="391"/>
+      <c r="O136" s="392"/>
+      <c r="Q136" s="390" t="s">
         <v>135</v>
       </c>
-      <c r="R136" s="358"/>
-      <c r="S136" s="359"/>
-      <c r="U136" s="357" t="s">
+      <c r="R136" s="391"/>
+      <c r="S136" s="392"/>
+      <c r="U136" s="390" t="s">
         <v>135</v>
       </c>
-      <c r="V136" s="358"/>
-      <c r="W136" s="359"/>
-      <c r="Y136" s="360" t="s">
+      <c r="V136" s="391"/>
+      <c r="W136" s="392"/>
+      <c r="Y136" s="398" t="s">
         <v>135</v>
       </c>
-      <c r="Z136" s="361"/>
-      <c r="AA136" s="361"/>
-      <c r="AB136" s="362"/>
+      <c r="Z136" s="399"/>
+      <c r="AA136" s="399"/>
+      <c r="AB136" s="400"/>
       <c r="AD136" s="160" t="s">
         <v>135</v>
       </c>
@@ -46745,32 +47631,32 @@
       <c r="G137" s="28" t="s">
         <v>101</v>
       </c>
-      <c r="M137" s="355">
+      <c r="M137" s="393">
         <v>6</v>
       </c>
-      <c r="N137" s="356"/>
+      <c r="N137" s="394"/>
       <c r="O137" s="111" t="s">
         <v>147</v>
       </c>
-      <c r="Q137" s="355">
+      <c r="Q137" s="393">
         <v>7</v>
       </c>
-      <c r="R137" s="356"/>
+      <c r="R137" s="394"/>
       <c r="S137" s="111" t="s">
         <v>147</v>
       </c>
-      <c r="U137" s="355">
+      <c r="U137" s="393">
         <v>8</v>
       </c>
-      <c r="V137" s="356"/>
+      <c r="V137" s="394"/>
       <c r="W137" s="111" t="s">
         <v>147</v>
       </c>
-      <c r="Y137" s="352">
+      <c r="Y137" s="395">
         <v>9</v>
       </c>
-      <c r="Z137" s="353"/>
-      <c r="AA137" s="354"/>
+      <c r="Z137" s="396"/>
+      <c r="AA137" s="397"/>
       <c r="AB137" s="198" t="s">
         <v>147</v>
       </c>
@@ -47877,35 +48763,35 @@
       <c r="L155" s="98" t="s">
         <v>191</v>
       </c>
-      <c r="M155" s="341" t="s">
+      <c r="M155" s="363" t="s">
         <v>206</v>
       </c>
-      <c r="N155" s="342"/>
-      <c r="O155" s="343"/>
+      <c r="N155" s="364"/>
+      <c r="O155" s="365"/>
       <c r="P155" s="98" t="s">
         <v>191</v>
       </c>
-      <c r="Q155" s="341" t="s">
+      <c r="Q155" s="363" t="s">
         <v>203</v>
       </c>
-      <c r="R155" s="342"/>
-      <c r="S155" s="343"/>
+      <c r="R155" s="364"/>
+      <c r="S155" s="365"/>
       <c r="T155" s="98" t="s">
         <v>191</v>
       </c>
-      <c r="U155" s="341" t="s">
+      <c r="U155" s="363" t="s">
         <v>351</v>
       </c>
-      <c r="V155" s="342"/>
-      <c r="W155" s="343"/>
+      <c r="V155" s="364"/>
+      <c r="W155" s="365"/>
       <c r="X155" s="98" t="s">
         <v>191</v>
       </c>
-      <c r="Y155" s="341" t="s">
+      <c r="Y155" s="363" t="s">
         <v>353</v>
       </c>
-      <c r="Z155" s="342"/>
-      <c r="AA155" s="343"/>
+      <c r="Z155" s="364"/>
+      <c r="AA155" s="365"/>
       <c r="AC155" s="98" t="s">
         <v>191</v>
       </c>
@@ -48085,38 +48971,38 @@
       </c>
     </row>
     <row r="174" spans="11:14" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="K174" s="375" t="s">
+      <c r="K174" s="378" t="s">
         <v>207</v>
       </c>
-      <c r="L174" s="376"/>
+      <c r="L174" s="379"/>
       <c r="M174" s="108">
         <f>O140+S140+W140+AB140+AF140</f>
         <v>1039</v>
       </c>
     </row>
     <row r="175" spans="11:14" x14ac:dyDescent="0.2">
-      <c r="K175" s="367" t="s">
+      <c r="K175" s="388" t="s">
         <v>196</v>
       </c>
-      <c r="L175" s="368"/>
+      <c r="L175" s="389"/>
       <c r="M175" s="108">
         <v>400</v>
       </c>
     </row>
     <row r="176" spans="11:14" x14ac:dyDescent="0.2">
-      <c r="K176" s="367" t="s">
+      <c r="K176" s="388" t="s">
         <v>359</v>
       </c>
-      <c r="L176" s="368"/>
+      <c r="L176" s="389"/>
       <c r="M176" s="109">
         <v>1312</v>
       </c>
     </row>
     <row r="177" spans="11:13" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="K177" s="369" t="s">
+      <c r="K177" s="374" t="s">
         <v>205</v>
       </c>
-      <c r="L177" s="370"/>
+      <c r="L177" s="375"/>
       <c r="M177" s="110">
         <f>M106</f>
         <v>1165</v>
@@ -48216,75 +49102,75 @@
       </c>
     </row>
     <row r="208" spans="9:36" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="M208" s="341" t="s">
+      <c r="M208" s="363" t="s">
         <v>135</v>
       </c>
-      <c r="N208" s="342"/>
-      <c r="O208" s="342"/>
-      <c r="P208" s="343"/>
-      <c r="R208" s="341" t="s">
+      <c r="N208" s="364"/>
+      <c r="O208" s="364"/>
+      <c r="P208" s="365"/>
+      <c r="R208" s="363" t="s">
         <v>135</v>
       </c>
-      <c r="S208" s="342"/>
-      <c r="T208" s="342"/>
-      <c r="U208" s="343"/>
-      <c r="W208" s="341" t="s">
+      <c r="S208" s="364"/>
+      <c r="T208" s="364"/>
+      <c r="U208" s="365"/>
+      <c r="W208" s="363" t="s">
         <v>135</v>
       </c>
-      <c r="X208" s="342"/>
-      <c r="Y208" s="342"/>
-      <c r="Z208" s="343"/>
-      <c r="AB208" s="341" t="s">
+      <c r="X208" s="364"/>
+      <c r="Y208" s="364"/>
+      <c r="Z208" s="365"/>
+      <c r="AB208" s="363" t="s">
         <v>135</v>
       </c>
-      <c r="AC208" s="342"/>
-      <c r="AD208" s="342"/>
-      <c r="AE208" s="343"/>
-      <c r="AG208" s="341" t="s">
+      <c r="AC208" s="364"/>
+      <c r="AD208" s="364"/>
+      <c r="AE208" s="365"/>
+      <c r="AG208" s="363" t="s">
         <v>135</v>
       </c>
-      <c r="AH208" s="342"/>
-      <c r="AI208" s="342"/>
-      <c r="AJ208" s="343"/>
+      <c r="AH208" s="364"/>
+      <c r="AI208" s="364"/>
+      <c r="AJ208" s="365"/>
     </row>
     <row r="209" spans="2:36" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="M209" s="364">
+      <c r="M209" s="384">
         <v>10</v>
       </c>
-      <c r="N209" s="365"/>
-      <c r="O209" s="366"/>
+      <c r="N209" s="385"/>
+      <c r="O209" s="386"/>
       <c r="P209" s="111" t="s">
         <v>147</v>
       </c>
-      <c r="R209" s="364">
+      <c r="R209" s="384">
         <v>11</v>
       </c>
-      <c r="S209" s="365"/>
-      <c r="T209" s="366"/>
+      <c r="S209" s="385"/>
+      <c r="T209" s="386"/>
       <c r="U209" s="111" t="s">
         <v>147</v>
       </c>
-      <c r="W209" s="364">
+      <c r="W209" s="384">
         <v>12</v>
       </c>
-      <c r="X209" s="365"/>
-      <c r="Y209" s="366"/>
+      <c r="X209" s="385"/>
+      <c r="Y209" s="386"/>
       <c r="Z209" s="111" t="s">
         <v>147</v>
       </c>
-      <c r="AB209" s="364">
+      <c r="AB209" s="384">
         <v>13</v>
       </c>
-      <c r="AC209" s="365"/>
-      <c r="AD209" s="366"/>
+      <c r="AC209" s="385"/>
+      <c r="AD209" s="386"/>
       <c r="AE209" s="111" t="s">
         <v>147</v>
       </c>
-      <c r="AG209" s="341">
-        <v>0</v>
-      </c>
-      <c r="AH209" s="342"/>
-      <c r="AI209" s="363"/>
+      <c r="AG209" s="363">
+        <v>0</v>
+      </c>
+      <c r="AH209" s="364"/>
+      <c r="AI209" s="387"/>
       <c r="AJ209" s="198" t="s">
         <v>147</v>
       </c>
@@ -49636,39 +50522,39 @@
       <c r="L227" s="98" t="s">
         <v>191</v>
       </c>
-      <c r="M227" s="341" t="s">
+      <c r="M227" s="363" t="s">
         <v>374</v>
       </c>
-      <c r="N227" s="342"/>
-      <c r="O227" s="343"/>
+      <c r="N227" s="364"/>
+      <c r="O227" s="365"/>
       <c r="Q227" s="98" t="s">
         <v>191</v>
       </c>
-      <c r="R227" s="341" t="s">
+      <c r="R227" s="363" t="s">
         <v>352</v>
       </c>
-      <c r="S227" s="342"/>
-      <c r="T227" s="343"/>
+      <c r="S227" s="364"/>
+      <c r="T227" s="365"/>
       <c r="V227" s="98" t="s">
         <v>191</v>
       </c>
-      <c r="W227" s="341"/>
-      <c r="X227" s="342"/>
-      <c r="Y227" s="343"/>
+      <c r="W227" s="363"/>
+      <c r="X227" s="364"/>
+      <c r="Y227" s="365"/>
       <c r="AA227" s="98" t="s">
         <v>191</v>
       </c>
-      <c r="AB227" s="341" t="s">
+      <c r="AB227" s="363" t="s">
         <v>409</v>
       </c>
-      <c r="AC227" s="342"/>
-      <c r="AD227" s="343"/>
+      <c r="AC227" s="364"/>
+      <c r="AD227" s="365"/>
       <c r="AF227" s="98" t="s">
         <v>191</v>
       </c>
-      <c r="AG227" s="341"/>
-      <c r="AH227" s="342"/>
-      <c r="AI227" s="343"/>
+      <c r="AG227" s="363"/>
+      <c r="AH227" s="364"/>
+      <c r="AI227" s="365"/>
     </row>
     <row r="228" spans="11:36" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="229" spans="11:36" ht="16" thickBot="1" x14ac:dyDescent="0.25">
@@ -49842,46 +50728,46 @@
       </c>
     </row>
     <row r="246" spans="11:14" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="K246" s="377" t="s">
+      <c r="K246" s="376" t="s">
         <v>207</v>
       </c>
-      <c r="L246" s="378"/>
+      <c r="L246" s="377"/>
       <c r="M246" s="108">
         <v>1039</v>
       </c>
     </row>
     <row r="247" spans="11:14" x14ac:dyDescent="0.2">
-      <c r="K247" s="375" t="s">
+      <c r="K247" s="378" t="s">
         <v>196</v>
       </c>
-      <c r="L247" s="376"/>
+      <c r="L247" s="379"/>
       <c r="M247" s="108">
         <v>400</v>
       </c>
     </row>
     <row r="248" spans="11:14" x14ac:dyDescent="0.2">
-      <c r="K248" s="373" t="s">
+      <c r="K248" s="380" t="s">
         <v>359</v>
       </c>
-      <c r="L248" s="374"/>
+      <c r="L248" s="381"/>
       <c r="M248" s="109">
         <v>1312</v>
       </c>
     </row>
     <row r="249" spans="11:14" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="K249" s="371" t="s">
+      <c r="K249" s="382" t="s">
         <v>205</v>
       </c>
-      <c r="L249" s="372"/>
+      <c r="L249" s="383"/>
       <c r="M249" s="110">
         <v>1165</v>
       </c>
     </row>
     <row r="250" spans="11:14" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="K250" s="369" t="s">
+      <c r="K250" s="374" t="s">
         <v>336</v>
       </c>
-      <c r="L250" s="370"/>
+      <c r="L250" s="375"/>
       <c r="M250" s="110">
         <f>P212+U212+Z212+AE212+AJ212</f>
         <v>730</v>
@@ -49984,75 +50870,75 @@
       </c>
     </row>
     <row r="280" spans="2:36" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="M280" s="341" t="s">
+      <c r="M280" s="363" t="s">
         <v>135</v>
       </c>
-      <c r="N280" s="342"/>
-      <c r="O280" s="342"/>
-      <c r="P280" s="343"/>
-      <c r="R280" s="341" t="s">
+      <c r="N280" s="364"/>
+      <c r="O280" s="364"/>
+      <c r="P280" s="365"/>
+      <c r="R280" s="363" t="s">
         <v>135</v>
       </c>
-      <c r="S280" s="342"/>
-      <c r="T280" s="342"/>
-      <c r="U280" s="343"/>
-      <c r="W280" s="341" t="s">
+      <c r="S280" s="364"/>
+      <c r="T280" s="364"/>
+      <c r="U280" s="365"/>
+      <c r="W280" s="363" t="s">
         <v>135</v>
       </c>
-      <c r="X280" s="342"/>
-      <c r="Y280" s="342"/>
-      <c r="Z280" s="343"/>
-      <c r="AB280" s="341" t="s">
+      <c r="X280" s="364"/>
+      <c r="Y280" s="364"/>
+      <c r="Z280" s="365"/>
+      <c r="AB280" s="363" t="s">
         <v>135</v>
       </c>
-      <c r="AC280" s="342"/>
-      <c r="AD280" s="342"/>
-      <c r="AE280" s="343"/>
-      <c r="AG280" s="341" t="s">
+      <c r="AC280" s="364"/>
+      <c r="AD280" s="364"/>
+      <c r="AE280" s="365"/>
+      <c r="AG280" s="363" t="s">
         <v>135</v>
       </c>
-      <c r="AH280" s="342"/>
-      <c r="AI280" s="342"/>
-      <c r="AJ280" s="343"/>
+      <c r="AH280" s="364"/>
+      <c r="AI280" s="364"/>
+      <c r="AJ280" s="365"/>
     </row>
     <row r="281" spans="2:36" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="M281" s="364">
+      <c r="M281" s="384">
         <v>14</v>
       </c>
-      <c r="N281" s="365"/>
-      <c r="O281" s="366"/>
+      <c r="N281" s="385"/>
+      <c r="O281" s="386"/>
       <c r="P281" s="111" t="s">
         <v>147</v>
       </c>
-      <c r="R281" s="364">
+      <c r="R281" s="384">
         <v>15</v>
       </c>
-      <c r="S281" s="365"/>
-      <c r="T281" s="366"/>
+      <c r="S281" s="385"/>
+      <c r="T281" s="386"/>
       <c r="U281" s="111" t="s">
         <v>147</v>
       </c>
-      <c r="W281" s="364">
+      <c r="W281" s="384">
         <v>16</v>
       </c>
-      <c r="X281" s="365"/>
-      <c r="Y281" s="366"/>
+      <c r="X281" s="385"/>
+      <c r="Y281" s="386"/>
       <c r="Z281" s="111" t="s">
         <v>147</v>
       </c>
-      <c r="AB281" s="364">
+      <c r="AB281" s="384">
         <v>17</v>
       </c>
-      <c r="AC281" s="365"/>
-      <c r="AD281" s="366"/>
+      <c r="AC281" s="385"/>
+      <c r="AD281" s="386"/>
       <c r="AE281" s="111" t="s">
         <v>147</v>
       </c>
-      <c r="AG281" s="341">
+      <c r="AG281" s="363">
         <v>18</v>
       </c>
-      <c r="AH281" s="342"/>
-      <c r="AI281" s="363"/>
+      <c r="AH281" s="364"/>
+      <c r="AI281" s="387"/>
       <c r="AJ281" s="198" t="s">
         <v>147</v>
       </c>
@@ -51370,39 +52256,39 @@
       <c r="L299" s="98" t="s">
         <v>191</v>
       </c>
-      <c r="M299" s="341" t="s">
+      <c r="M299" s="363" t="s">
         <v>374</v>
       </c>
-      <c r="N299" s="342"/>
-      <c r="O299" s="343"/>
+      <c r="N299" s="364"/>
+      <c r="O299" s="365"/>
       <c r="Q299" s="98" t="s">
         <v>191</v>
       </c>
-      <c r="R299" s="341" t="s">
+      <c r="R299" s="363" t="s">
         <v>352</v>
       </c>
-      <c r="S299" s="342"/>
-      <c r="T299" s="343"/>
+      <c r="S299" s="364"/>
+      <c r="T299" s="365"/>
       <c r="V299" s="98" t="s">
         <v>191</v>
       </c>
-      <c r="W299" s="341"/>
-      <c r="X299" s="342"/>
-      <c r="Y299" s="343"/>
+      <c r="W299" s="363"/>
+      <c r="X299" s="364"/>
+      <c r="Y299" s="365"/>
       <c r="AA299" s="98" t="s">
         <v>191</v>
       </c>
-      <c r="AB299" s="341" t="s">
+      <c r="AB299" s="363" t="s">
         <v>409</v>
       </c>
-      <c r="AC299" s="342"/>
-      <c r="AD299" s="343"/>
+      <c r="AC299" s="364"/>
+      <c r="AD299" s="365"/>
       <c r="AF299" s="98" t="s">
         <v>191</v>
       </c>
-      <c r="AG299" s="341"/>
-      <c r="AH299" s="342"/>
-      <c r="AI299" s="343"/>
+      <c r="AG299" s="363"/>
+      <c r="AH299" s="364"/>
+      <c r="AI299" s="365"/>
     </row>
     <row r="300" spans="2:36" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="301" spans="2:36" ht="16" thickBot="1" x14ac:dyDescent="0.25">
@@ -51579,10 +52465,10 @@
       </c>
     </row>
     <row r="318" spans="11:14" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="K318" s="377" t="s">
+      <c r="K318" s="376" t="s">
         <v>207</v>
       </c>
-      <c r="L318" s="378"/>
+      <c r="L318" s="377"/>
       <c r="M318" s="253">
         <v>1039</v>
       </c>
@@ -51592,20 +52478,20 @@
       </c>
     </row>
     <row r="319" spans="11:14" x14ac:dyDescent="0.2">
-      <c r="K319" s="375" t="s">
+      <c r="K319" s="378" t="s">
         <v>196</v>
       </c>
-      <c r="L319" s="376"/>
+      <c r="L319" s="379"/>
       <c r="M319" s="253">
         <v>400</v>
       </c>
       <c r="N319" s="257"/>
     </row>
     <row r="320" spans="11:14" x14ac:dyDescent="0.2">
-      <c r="K320" s="373" t="s">
+      <c r="K320" s="380" t="s">
         <v>359</v>
       </c>
-      <c r="L320" s="374"/>
+      <c r="L320" s="381"/>
       <c r="M320" s="254">
         <v>1312</v>
       </c>
@@ -51615,10 +52501,10 @@
       </c>
     </row>
     <row r="321" spans="11:15" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="K321" s="371" t="s">
+      <c r="K321" s="382" t="s">
         <v>205</v>
       </c>
-      <c r="L321" s="372"/>
+      <c r="L321" s="383"/>
       <c r="M321" s="255">
         <v>1165</v>
       </c>
@@ -51628,10 +52514,10 @@
       </c>
     </row>
     <row r="322" spans="11:15" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="K322" s="369" t="s">
+      <c r="K322" s="374" t="s">
         <v>336</v>
       </c>
-      <c r="L322" s="370"/>
+      <c r="L322" s="375"/>
       <c r="M322" s="255">
         <f>M250</f>
         <v>730</v>
@@ -51645,10 +52531,10 @@
       </c>
     </row>
     <row r="323" spans="11:15" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="K323" s="369" t="s">
+      <c r="K323" s="374" t="s">
         <v>421</v>
       </c>
-      <c r="L323" s="370"/>
+      <c r="L323" s="375"/>
       <c r="M323" s="255">
         <f>P284+U284+Z284+AE284+AJ284</f>
         <v>1054</v>
@@ -51774,75 +52660,75 @@
       </c>
     </row>
     <row r="352" spans="2:36" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="M352" s="341" t="s">
+      <c r="M352" s="363" t="s">
         <v>135</v>
       </c>
-      <c r="N352" s="342"/>
-      <c r="O352" s="342"/>
-      <c r="P352" s="343"/>
-      <c r="R352" s="341" t="s">
+      <c r="N352" s="364"/>
+      <c r="O352" s="364"/>
+      <c r="P352" s="365"/>
+      <c r="R352" s="363" t="s">
         <v>135</v>
       </c>
-      <c r="S352" s="342"/>
-      <c r="T352" s="342"/>
-      <c r="U352" s="343"/>
-      <c r="W352" s="341" t="s">
+      <c r="S352" s="364"/>
+      <c r="T352" s="364"/>
+      <c r="U352" s="365"/>
+      <c r="W352" s="363" t="s">
         <v>135</v>
       </c>
-      <c r="X352" s="342"/>
-      <c r="Y352" s="342"/>
-      <c r="Z352" s="343"/>
-      <c r="AB352" s="341" t="s">
+      <c r="X352" s="364"/>
+      <c r="Y352" s="364"/>
+      <c r="Z352" s="365"/>
+      <c r="AB352" s="363" t="s">
         <v>135</v>
       </c>
-      <c r="AC352" s="342"/>
-      <c r="AD352" s="342"/>
-      <c r="AE352" s="343"/>
-      <c r="AG352" s="341" t="s">
+      <c r="AC352" s="364"/>
+      <c r="AD352" s="364"/>
+      <c r="AE352" s="365"/>
+      <c r="AG352" s="363" t="s">
         <v>135</v>
       </c>
-      <c r="AH352" s="342"/>
-      <c r="AI352" s="342"/>
-      <c r="AJ352" s="343"/>
+      <c r="AH352" s="364"/>
+      <c r="AI352" s="364"/>
+      <c r="AJ352" s="365"/>
     </row>
     <row r="353" spans="2:36" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="M353" s="364">
+      <c r="M353" s="384">
         <v>27</v>
       </c>
-      <c r="N353" s="365"/>
-      <c r="O353" s="366"/>
+      <c r="N353" s="385"/>
+      <c r="O353" s="386"/>
       <c r="P353" s="111" t="s">
         <v>147</v>
       </c>
-      <c r="R353" s="364">
+      <c r="R353" s="384">
         <v>28</v>
       </c>
-      <c r="S353" s="365"/>
-      <c r="T353" s="366"/>
+      <c r="S353" s="385"/>
+      <c r="T353" s="386"/>
       <c r="U353" s="111" t="s">
         <v>147</v>
       </c>
-      <c r="W353" s="364">
+      <c r="W353" s="384">
         <v>29</v>
       </c>
-      <c r="X353" s="365"/>
-      <c r="Y353" s="366"/>
+      <c r="X353" s="385"/>
+      <c r="Y353" s="386"/>
       <c r="Z353" s="111" t="s">
         <v>147</v>
       </c>
-      <c r="AB353" s="364">
+      <c r="AB353" s="384">
         <v>30</v>
       </c>
-      <c r="AC353" s="365"/>
-      <c r="AD353" s="366"/>
+      <c r="AC353" s="385"/>
+      <c r="AD353" s="386"/>
       <c r="AE353" s="111" t="s">
         <v>147</v>
       </c>
-      <c r="AG353" s="341">
+      <c r="AG353" s="363">
         <v>31</v>
       </c>
-      <c r="AH353" s="342"/>
-      <c r="AI353" s="363"/>
+      <c r="AH353" s="364"/>
+      <c r="AI353" s="387"/>
       <c r="AJ353" s="198" t="s">
         <v>147</v>
       </c>
@@ -53038,33 +53924,33 @@
       <c r="L371" s="98" t="s">
         <v>191</v>
       </c>
-      <c r="M371" s="341"/>
-      <c r="N371" s="342"/>
-      <c r="O371" s="343"/>
+      <c r="M371" s="363"/>
+      <c r="N371" s="364"/>
+      <c r="O371" s="365"/>
       <c r="Q371" s="98" t="s">
         <v>191</v>
       </c>
-      <c r="R371" s="341"/>
-      <c r="S371" s="342"/>
-      <c r="T371" s="343"/>
+      <c r="R371" s="363"/>
+      <c r="S371" s="364"/>
+      <c r="T371" s="365"/>
       <c r="V371" s="98" t="s">
         <v>191</v>
       </c>
-      <c r="W371" s="341"/>
-      <c r="X371" s="342"/>
-      <c r="Y371" s="343"/>
+      <c r="W371" s="363"/>
+      <c r="X371" s="364"/>
+      <c r="Y371" s="365"/>
       <c r="AA371" s="98" t="s">
         <v>191</v>
       </c>
-      <c r="AB371" s="341"/>
-      <c r="AC371" s="342"/>
-      <c r="AD371" s="343"/>
+      <c r="AB371" s="363"/>
+      <c r="AC371" s="364"/>
+      <c r="AD371" s="365"/>
       <c r="AF371" s="98" t="s">
         <v>191</v>
       </c>
-      <c r="AG371" s="341"/>
-      <c r="AH371" s="342"/>
-      <c r="AI371" s="343"/>
+      <c r="AG371" s="363"/>
+      <c r="AH371" s="364"/>
+      <c r="AI371" s="365"/>
     </row>
     <row r="372" spans="11:36" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="373" spans="11:36" ht="16" thickBot="1" x14ac:dyDescent="0.25">
@@ -53241,10 +54127,10 @@
       </c>
     </row>
     <row r="390" spans="11:15" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="K390" s="377" t="s">
+      <c r="K390" s="376" t="s">
         <v>207</v>
       </c>
-      <c r="L390" s="378"/>
+      <c r="L390" s="377"/>
       <c r="M390" s="253">
         <v>1039</v>
       </c>
@@ -53254,20 +54140,20 @@
       </c>
     </row>
     <row r="391" spans="11:15" x14ac:dyDescent="0.2">
-      <c r="K391" s="375" t="s">
+      <c r="K391" s="378" t="s">
         <v>196</v>
       </c>
-      <c r="L391" s="376"/>
+      <c r="L391" s="379"/>
       <c r="M391" s="253">
         <v>400</v>
       </c>
       <c r="N391" s="257"/>
     </row>
     <row r="392" spans="11:15" x14ac:dyDescent="0.2">
-      <c r="K392" s="373" t="s">
+      <c r="K392" s="380" t="s">
         <v>359</v>
       </c>
-      <c r="L392" s="374"/>
+      <c r="L392" s="381"/>
       <c r="M392" s="254">
         <v>1312</v>
       </c>
@@ -53277,10 +54163,10 @@
       </c>
     </row>
     <row r="393" spans="11:15" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="K393" s="371" t="s">
+      <c r="K393" s="382" t="s">
         <v>205</v>
       </c>
-      <c r="L393" s="372"/>
+      <c r="L393" s="383"/>
       <c r="M393" s="255">
         <v>1165</v>
       </c>
@@ -53290,10 +54176,10 @@
       </c>
     </row>
     <row r="394" spans="11:15" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="K394" s="369" t="s">
+      <c r="K394" s="374" t="s">
         <v>336</v>
       </c>
-      <c r="L394" s="370"/>
+      <c r="L394" s="375"/>
       <c r="M394" s="255">
         <f>M322</f>
         <v>730</v>
@@ -53307,10 +54193,10 @@
       </c>
     </row>
     <row r="395" spans="11:15" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="K395" s="369" t="s">
+      <c r="K395" s="374" t="s">
         <v>421</v>
       </c>
-      <c r="L395" s="370"/>
+      <c r="L395" s="375"/>
       <c r="M395" s="255">
         <f>P356+U356+Z356+AE356+AJ356</f>
         <v>130</v>
@@ -53328,68 +54214,23 @@
     <sortCondition descending="1" ref="L31:L38"/>
   </sortState>
   <mergeCells count="103">
-    <mergeCell ref="K395:L395"/>
-    <mergeCell ref="K390:L390"/>
-    <mergeCell ref="K391:L391"/>
-    <mergeCell ref="K392:L392"/>
-    <mergeCell ref="K393:L393"/>
-    <mergeCell ref="K394:L394"/>
-    <mergeCell ref="M371:O371"/>
-    <mergeCell ref="R371:T371"/>
-    <mergeCell ref="W371:Y371"/>
-    <mergeCell ref="AB371:AD371"/>
-    <mergeCell ref="AG371:AI371"/>
-    <mergeCell ref="M353:O353"/>
-    <mergeCell ref="R353:T353"/>
-    <mergeCell ref="W353:Y353"/>
-    <mergeCell ref="AB353:AD353"/>
-    <mergeCell ref="AG353:AI353"/>
-    <mergeCell ref="M352:P352"/>
-    <mergeCell ref="R352:U352"/>
-    <mergeCell ref="W352:Z352"/>
-    <mergeCell ref="AB352:AE352"/>
-    <mergeCell ref="AG352:AJ352"/>
-    <mergeCell ref="K323:L323"/>
-    <mergeCell ref="AG280:AJ280"/>
-    <mergeCell ref="AB280:AE280"/>
-    <mergeCell ref="W280:Z280"/>
-    <mergeCell ref="R280:U280"/>
-    <mergeCell ref="M280:P280"/>
-    <mergeCell ref="AG281:AI281"/>
-    <mergeCell ref="AB281:AD281"/>
-    <mergeCell ref="W281:Y281"/>
-    <mergeCell ref="R281:T281"/>
-    <mergeCell ref="M281:O281"/>
-    <mergeCell ref="AG299:AI299"/>
-    <mergeCell ref="AB299:AD299"/>
-    <mergeCell ref="W299:Y299"/>
-    <mergeCell ref="R299:T299"/>
-    <mergeCell ref="M299:O299"/>
-    <mergeCell ref="K322:L322"/>
-    <mergeCell ref="K321:L321"/>
-    <mergeCell ref="K320:L320"/>
-    <mergeCell ref="K319:L319"/>
-    <mergeCell ref="K318:L318"/>
-    <mergeCell ref="K250:L250"/>
-    <mergeCell ref="K249:L249"/>
-    <mergeCell ref="K248:L248"/>
-    <mergeCell ref="K175:L175"/>
-    <mergeCell ref="K174:L174"/>
-    <mergeCell ref="K246:L246"/>
-    <mergeCell ref="K247:L247"/>
-    <mergeCell ref="K176:L176"/>
-    <mergeCell ref="K177:L177"/>
-    <mergeCell ref="AC66:AE66"/>
-    <mergeCell ref="AC67:AD67"/>
-    <mergeCell ref="AC85:AE85"/>
-    <mergeCell ref="Y85:AA85"/>
-    <mergeCell ref="M66:O66"/>
-    <mergeCell ref="Q66:S66"/>
-    <mergeCell ref="U66:W66"/>
-    <mergeCell ref="Y66:AA66"/>
-    <mergeCell ref="M67:N67"/>
-    <mergeCell ref="Q67:R67"/>
-    <mergeCell ref="U67:V67"/>
+    <mergeCell ref="Y137:AA137"/>
+    <mergeCell ref="Y67:Z67"/>
+    <mergeCell ref="M136:O136"/>
+    <mergeCell ref="Q136:S136"/>
+    <mergeCell ref="U136:W136"/>
+    <mergeCell ref="Y136:AB136"/>
+    <mergeCell ref="AG227:AI227"/>
+    <mergeCell ref="AG208:AJ208"/>
+    <mergeCell ref="AB208:AE208"/>
+    <mergeCell ref="W208:Z208"/>
+    <mergeCell ref="R208:U208"/>
+    <mergeCell ref="AG209:AI209"/>
+    <mergeCell ref="W209:Y209"/>
+    <mergeCell ref="AB209:AD209"/>
+    <mergeCell ref="R227:T227"/>
+    <mergeCell ref="W227:Y227"/>
+    <mergeCell ref="AB227:AD227"/>
     <mergeCell ref="K105:L105"/>
     <mergeCell ref="K106:L106"/>
     <mergeCell ref="M85:O85"/>
@@ -53414,23 +54255,68 @@
     <mergeCell ref="M137:N137"/>
     <mergeCell ref="Q137:R137"/>
     <mergeCell ref="U137:V137"/>
-    <mergeCell ref="Y137:AA137"/>
-    <mergeCell ref="Y67:Z67"/>
-    <mergeCell ref="M136:O136"/>
-    <mergeCell ref="Q136:S136"/>
-    <mergeCell ref="U136:W136"/>
-    <mergeCell ref="Y136:AB136"/>
-    <mergeCell ref="AG227:AI227"/>
-    <mergeCell ref="AG208:AJ208"/>
-    <mergeCell ref="AB208:AE208"/>
-    <mergeCell ref="W208:Z208"/>
-    <mergeCell ref="R208:U208"/>
-    <mergeCell ref="AG209:AI209"/>
-    <mergeCell ref="W209:Y209"/>
-    <mergeCell ref="AB209:AD209"/>
-    <mergeCell ref="R227:T227"/>
-    <mergeCell ref="W227:Y227"/>
-    <mergeCell ref="AB227:AD227"/>
+    <mergeCell ref="AC66:AE66"/>
+    <mergeCell ref="AC67:AD67"/>
+    <mergeCell ref="AC85:AE85"/>
+    <mergeCell ref="Y85:AA85"/>
+    <mergeCell ref="M66:O66"/>
+    <mergeCell ref="Q66:S66"/>
+    <mergeCell ref="U66:W66"/>
+    <mergeCell ref="Y66:AA66"/>
+    <mergeCell ref="M67:N67"/>
+    <mergeCell ref="Q67:R67"/>
+    <mergeCell ref="U67:V67"/>
+    <mergeCell ref="K250:L250"/>
+    <mergeCell ref="K249:L249"/>
+    <mergeCell ref="K248:L248"/>
+    <mergeCell ref="K175:L175"/>
+    <mergeCell ref="K174:L174"/>
+    <mergeCell ref="K246:L246"/>
+    <mergeCell ref="K247:L247"/>
+    <mergeCell ref="K176:L176"/>
+    <mergeCell ref="K177:L177"/>
+    <mergeCell ref="K323:L323"/>
+    <mergeCell ref="AG280:AJ280"/>
+    <mergeCell ref="AB280:AE280"/>
+    <mergeCell ref="W280:Z280"/>
+    <mergeCell ref="R280:U280"/>
+    <mergeCell ref="M280:P280"/>
+    <mergeCell ref="AG281:AI281"/>
+    <mergeCell ref="AB281:AD281"/>
+    <mergeCell ref="W281:Y281"/>
+    <mergeCell ref="R281:T281"/>
+    <mergeCell ref="M281:O281"/>
+    <mergeCell ref="AG299:AI299"/>
+    <mergeCell ref="AB299:AD299"/>
+    <mergeCell ref="W299:Y299"/>
+    <mergeCell ref="R299:T299"/>
+    <mergeCell ref="M299:O299"/>
+    <mergeCell ref="K322:L322"/>
+    <mergeCell ref="K321:L321"/>
+    <mergeCell ref="K320:L320"/>
+    <mergeCell ref="K319:L319"/>
+    <mergeCell ref="K318:L318"/>
+    <mergeCell ref="AB371:AD371"/>
+    <mergeCell ref="AG371:AI371"/>
+    <mergeCell ref="M353:O353"/>
+    <mergeCell ref="R353:T353"/>
+    <mergeCell ref="W353:Y353"/>
+    <mergeCell ref="AB353:AD353"/>
+    <mergeCell ref="AG353:AI353"/>
+    <mergeCell ref="M352:P352"/>
+    <mergeCell ref="R352:U352"/>
+    <mergeCell ref="W352:Z352"/>
+    <mergeCell ref="AB352:AE352"/>
+    <mergeCell ref="AG352:AJ352"/>
+    <mergeCell ref="K395:L395"/>
+    <mergeCell ref="K390:L390"/>
+    <mergeCell ref="K391:L391"/>
+    <mergeCell ref="K392:L392"/>
+    <mergeCell ref="K393:L393"/>
+    <mergeCell ref="K394:L394"/>
+    <mergeCell ref="M371:O371"/>
+    <mergeCell ref="R371:T371"/>
+    <mergeCell ref="W371:Y371"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Fly Deltoid N2 → delts + traps
Confirmed reverse fly machine; mapping now matches Rear Deltoid N1.
</commit_message>
<xml_diff>
--- a/My Lattice&Climbing training docs/Jo_training raw docs 25_2026/myGym Training 24_2025.xlsx
+++ b/My Lattice&Climbing training docs/Jo_training raw docs 25_2026/myGym Training 24_2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/josinabernardes/Documents/Tennis-Tracker-Hub/My Lattice&amp;Climbing training docs/Jo_training raw docs 25_2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51EE60B5-5420-874F-9FBF-D6EB1779B797}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D935A34E-58CC-F64C-86E7-F898DBCD3BF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4320" yWindow="600" windowWidth="24480" windowHeight="15940" tabRatio="765" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40316,8 +40316,8 @@
         <v>27</v>
       </c>
       <c r="M38" s="42">
-        <f>M33</f>
-        <v>51.5</v>
+        <f>M33+(K38+L38)</f>
+        <v>78.5</v>
       </c>
       <c r="N38" s="126" t="s">
         <v>218</v>
@@ -40408,8 +40408,8 @@
         <v>0</v>
       </c>
       <c r="M41" s="42">
-        <f>M33</f>
-        <v>51.5</v>
+        <f>M33+(K41+L41)</f>
+        <v>28.5</v>
       </c>
       <c r="N41" s="126" t="s">
         <v>218</v>
@@ -40500,8 +40500,8 @@
         <v>42</v>
       </c>
       <c r="M44" s="42">
-        <f>M33</f>
-        <v>51.5</v>
+        <f>M33+(K44+L44)</f>
+        <v>93.5</v>
       </c>
       <c r="N44" s="126" t="s">
         <v>218</v>
@@ -40598,8 +40598,8 @@
         <v>7</v>
       </c>
       <c r="M48" s="42">
-        <f>M33</f>
-        <v>51.5</v>
+        <f>M33+(K48+L48)</f>
+        <v>58.5</v>
       </c>
       <c r="N48" s="126" t="s">
         <v>218</v>
@@ -40689,8 +40689,8 @@
         <v>13.5</v>
       </c>
       <c r="M51" s="42">
-        <f>M33</f>
-        <v>51.5</v>
+        <f>M33+(K51+L51)</f>
+        <v>65</v>
       </c>
       <c r="N51" s="126" t="s">
         <v>218</v>
@@ -40780,8 +40780,8 @@
         <v>13.5</v>
       </c>
       <c r="M54" s="42">
-        <f>M5</f>
-        <v>0</v>
+        <f>M33+(K54+L54)</f>
+        <v>65</v>
       </c>
       <c r="N54" s="126" t="s">
         <v>218</v>
@@ -40871,8 +40871,8 @@
         <v>13.5</v>
       </c>
       <c r="M57" s="42">
-        <f>M33</f>
-        <v>51.5</v>
+        <f>M33+(K57+L57)</f>
+        <v>65</v>
       </c>
       <c r="N57" s="126" t="s">
         <v>218</v>
@@ -40962,8 +40962,8 @@
         <v>13.5</v>
       </c>
       <c r="M60" s="42">
-        <f>M33</f>
-        <v>51.5</v>
+        <f>M33+(K60+L60)</f>
+        <v>65</v>
       </c>
       <c r="N60" s="126" t="s">
         <v>218</v>

</xml_diff>